<commit_message>
update: extend xlsx tests and argument unit tests for TIME, HOUR, MINUTE, SECOND
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/DATE_AND_TIME/TIME_HOUR_MINUTE_SECOND.xlsx
+++ b/xlsx/tests/calc_tests/DATE_AND_TIME/TIME_HOUR_MINUTE_SECOND.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29429"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhatcher/Documents/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elsam\Documents\IronCalc stuff\my_calc_tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBC0634F-134E-41A2-B667-6435048C259E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A35D429E-2E32-4024-9948-77450FEAF236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33600" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{F5EF1803-C89D-8542-8C3F-E05EFF447D52}"/>
+    <workbookView xWindow="5990" yWindow="3860" windowWidth="28800" windowHeight="15290" xr2:uid="{F5EF1803-C89D-8542-8C3F-E05EFF447D52}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,8 +35,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="60">
   <si>
     <t>HOUR</t>
   </si>
@@ -111,6 +133,111 @@
   </si>
   <si>
     <t>Boolean as input</t>
+  </si>
+  <si>
+    <t>Hours beyond the 32767 bound</t>
+  </si>
+  <si>
+    <t>Minutes beyond the 32767 bound</t>
+  </si>
+  <si>
+    <t>Seconds beyond the 32767 bound</t>
+  </si>
+  <si>
+    <t>One argument beyond bound, others at bound</t>
+  </si>
+  <si>
+    <t>All arguments zero</t>
+  </si>
+  <si>
+    <t>Smallest non-zero time</t>
+  </si>
+  <si>
+    <t>Largest time within one day</t>
+  </si>
+  <si>
+    <t>Seconds roll over into the next day</t>
+  </si>
+  <si>
+    <t>Seconds equal to one day minus one</t>
+  </si>
+  <si>
+    <t>Seconds equal to exactly one day</t>
+  </si>
+  <si>
+    <t>Seconds just beyond one day</t>
+  </si>
+  <si>
+    <t>Minutes equal to exactly one day</t>
+  </si>
+  <si>
+    <t>Hours equal to exactly one day</t>
+  </si>
+  <si>
+    <t>Hours equal to exactly two days</t>
+  </si>
+  <si>
+    <t>All arguments negative</t>
+  </si>
+  <si>
+    <t>Negative seconds from midnight</t>
+  </si>
+  <si>
+    <t>Negative minutes from midnight</t>
+  </si>
+  <si>
+    <t>Seconds fraction rounds down</t>
+  </si>
+  <si>
+    <t>Seconds fraction at the rounding midpoint</t>
+  </si>
+  <si>
+    <t>All arguments just above zero</t>
+  </si>
+  <si>
+    <t>Date with a time portion</t>
+  </si>
+  <si>
+    <t>Whole date, no time portion</t>
+  </si>
+  <si>
+    <t>Serial 0</t>
+  </si>
+  <si>
+    <t>Serial 0.5, exactly midday</t>
+  </si>
+  <si>
+    <t>Serial 0.25, 6am</t>
+  </si>
+  <si>
+    <t>Serial 1, exactly one day</t>
+  </si>
+  <si>
+    <t>Negative serial</t>
+  </si>
+  <si>
+    <t>Negative whole serial</t>
+  </si>
+  <si>
+    <t>Maximum date with a time portion</t>
+  </si>
+  <si>
+    <t>Serial beyond the maximum date</t>
+  </si>
+  <si>
+    <t>Serial just above one whole day</t>
+  </si>
+  <si>
+    <t>Boolean TRUE</t>
+  </si>
+  <si>
+    <t>Error propagation mixed</t>
+  </si>
+  <si>
+    <t>Negative near zero</t>
+  </si>
+  <si>
+    <t>All arguments negative near zero</t>
   </si>
 </sst>
 </file>
@@ -118,10 +245,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="0.0000000000"/>
-    <numFmt numFmtId="166" formatCode="h:mm:ss;@"/>
+    <numFmt numFmtId="164" formatCode="0.0000000000"/>
+    <numFmt numFmtId="165" formatCode="h:mm:ss;@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -153,6 +280,18 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -196,18 +335,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
@@ -541,10 +683,32 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="525" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{86F010F7-E038-4299-9ABC-6B7FD165E119}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;759a215b-68d0-4a32-b792-08a4fe5196a6&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4323771-C859-F046-B681-A08AFC84A35B}">
-  <dimension ref="A1:I36"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:I61"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.25" style="1" customWidth="1"/>
     <col min="2" max="3" width="11" style="1"/>
@@ -555,7 +719,7 @@
     <col min="10" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75">
+    <row r="1" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -581,7 +745,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>3</v>
       </c>
@@ -612,7 +776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>24</v>
       </c>
@@ -646,7 +810,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>16</v>
       </c>
@@ -661,7 +825,7 @@
         <v>0.70861111111111108</v>
       </c>
       <c r="E4" s="4">
-        <f t="shared" ref="E4:E26" si="1">D4</f>
+        <f t="shared" ref="E4:E24" si="1">D4</f>
         <v>0.70861111111111108</v>
       </c>
       <c r="F4" s="2">
@@ -680,7 +844,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>3.1</v>
       </c>
@@ -714,7 +878,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>23</v>
       </c>
@@ -748,7 +912,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="D7" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -773,7 +937,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>23</v>
       </c>
@@ -801,7 +965,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B9" s="1">
         <v>23</v>
       </c>
@@ -829,7 +993,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="C10" s="1">
         <v>23</v>
       </c>
@@ -857,7 +1021,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>-1</v>
       </c>
@@ -891,7 +1055,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>12</v>
       </c>
@@ -925,7 +1089,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>13</v>
       </c>
@@ -959,7 +1123,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>34</v>
       </c>
@@ -993,7 +1157,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>10</v>
       </c>
@@ -1027,7 +1191,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>10</v>
       </c>
@@ -1061,7 +1225,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A17" s="1">
         <v>32767</v>
       </c>
@@ -1095,7 +1259,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
@@ -1130,19 +1294,19 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A19" s="1">
         <v>1</v>
       </c>
       <c r="B19" s="1" t="e">
-        <f t="shared" ref="B19:C20" si="28">1/0</f>
+        <f t="shared" ref="B19:C21" si="28">1/0</f>
         <v>#DIV/0!</v>
       </c>
       <c r="C19" s="1">
         <v>3</v>
       </c>
       <c r="D19" s="7" t="e">
-        <f t="shared" ref="D19:D26" si="29">TIME(A19,B19,C19)</f>
+        <f t="shared" ref="D19:D24" si="29">TIME(A19,B19,C19)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="E19" s="4" t="e">
@@ -1150,22 +1314,22 @@
         <v>#DIV/0!</v>
       </c>
       <c r="F19" s="2" t="e">
-        <f t="shared" ref="F19:F23" si="30">HOUR(D19)</f>
+        <f t="shared" ref="F19:F21" si="30">HOUR(D19)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G19" s="2" t="e">
-        <f t="shared" ref="G19:G23" si="31">MINUTE(D19)</f>
+        <f t="shared" ref="G19:G21" si="31">MINUTE(D19)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="H19" s="2" t="e">
-        <f t="shared" ref="H19:H23" si="32">SECOND(D19)</f>
+        <f t="shared" ref="H19:H21" si="32">SECOND(D19)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A20" s="1">
         <v>1</v>
       </c>
@@ -1200,224 +1364,1146 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="B21" s="1">
-        <v>2</v>
-      </c>
-      <c r="C21" s="1">
-        <v>3</v>
+      <c r="B21" s="1" t="e">
+        <f t="shared" si="28"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C21" s="1" t="e" cm="1">
+        <f t="array" aca="1" ref="C21" ca="1">hello()</f>
+        <v>#NAME?</v>
       </c>
       <c r="D21" s="7" t="e">
+        <f t="shared" ca="1" si="29"/>
+        <v>#N/A</v>
+      </c>
+      <c r="E21" s="4" t="e">
+        <f t="shared" ca="1" si="1"/>
+        <v>#N/A</v>
+      </c>
+      <c r="F21" s="2" t="e">
+        <f t="shared" ca="1" si="30"/>
+        <v>#N/A</v>
+      </c>
+      <c r="G21" s="2" t="e">
+        <f t="shared" ca="1" si="31"/>
+        <v>#N/A</v>
+      </c>
+      <c r="H21" s="2" t="e">
+        <f t="shared" ca="1" si="32"/>
+        <v>#N/A</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="7" t="e">
         <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="E21" s="4" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E22" s="4" t="e">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="F21" s="2" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="G21" s="2" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H21" s="2" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" s="1">
-        <v>1</v>
-      </c>
-      <c r="B22" s="1" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F22" s="2" t="e">
+        <f t="shared" ref="F22" si="33">HOUR(D22)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G22" s="2" t="e">
+        <f t="shared" ref="G22" si="34">MINUTE(D22)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H22" s="2" t="e">
+        <f t="shared" ref="H22" si="35">SECOND(D22)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A23" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D23" s="7" t="e">
+        <f t="shared" si="29"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E23" s="4" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F23" s="2" t="e">
+        <f t="shared" ref="F23" si="36">HOUR(D23)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G23" s="2" t="e">
+        <f t="shared" ref="G23" si="37">MINUTE(D23)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H23" s="2" t="e">
+        <f t="shared" ref="H23" si="38">SECOND(D23)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="B24" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="C24" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D24" s="7">
+        <f t="shared" si="29"/>
+        <v>4.1678240740740738E-2</v>
+      </c>
+      <c r="E24" s="4">
+        <f t="shared" si="1"/>
+        <v>4.1678240740740738E-2</v>
+      </c>
+      <c r="F24" s="2">
+        <f t="shared" ref="F24" si="39">HOUR(D24)</f>
+        <v>1</v>
+      </c>
+      <c r="G24" s="2">
+        <f t="shared" ref="G24" si="40">MINUTE(D24)</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="2">
+        <f t="shared" ref="H24" si="41">SECOND(D24)</f>
+        <v>1</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="14.5" x14ac:dyDescent="0.35"/>
+    <row r="26" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A26" s="1">
+        <v>32768</v>
+      </c>
+      <c r="B26" s="1">
+        <v>1</v>
+      </c>
+      <c r="C26" s="1">
+        <v>1</v>
+      </c>
+      <c r="D26" s="7" t="e">
+        <f t="shared" ref="D26:D46" si="42">TIME(A26,B26,C26)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="E26" s="9" t="e">
+        <f t="shared" ref="E26:E46" si="43">D26</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="F26" s="2" t="e">
+        <f t="shared" ref="F26:F46" si="44">HOUR(D26)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="G26" s="2" t="e">
+        <f t="shared" ref="G26:G46" si="45">MINUTE(D26)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="H26" s="2" t="e">
+        <f t="shared" ref="H26:H46" si="46">SECOND(D26)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A27" s="1">
+        <v>1</v>
+      </c>
+      <c r="B27" s="1">
+        <v>32768</v>
+      </c>
+      <c r="C27" s="1">
+        <v>1</v>
+      </c>
+      <c r="D27" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E27" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F27" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G27" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H27" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A28" s="1">
+        <v>1</v>
+      </c>
+      <c r="B28" s="1">
+        <v>1</v>
+      </c>
+      <c r="C28" s="1">
+        <v>32768</v>
+      </c>
+      <c r="D28" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E28" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F28" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G28" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H28" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A29" s="1">
+        <v>32767</v>
+      </c>
+      <c r="B29" s="1">
+        <v>32767</v>
+      </c>
+      <c r="C29" s="1">
+        <v>32768</v>
+      </c>
+      <c r="D29" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E29" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F29" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G29" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H29" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A30" s="1">
+        <v>0</v>
+      </c>
+      <c r="B30" s="1">
+        <v>0</v>
+      </c>
+      <c r="C30" s="1">
+        <v>0</v>
+      </c>
+      <c r="D30" s="7">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="E30" s="9">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="F30" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G30" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H30" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A31" s="1">
+        <v>0</v>
+      </c>
+      <c r="B31" s="1">
+        <v>0</v>
+      </c>
+      <c r="C31" s="1">
+        <v>1</v>
+      </c>
+      <c r="D31" s="7">
+        <f t="shared" si="42"/>
+        <v>1.1574074074074073E-5</v>
+      </c>
+      <c r="E31" s="9">
+        <f t="shared" si="43"/>
+        <v>1.1574074074074073E-5</v>
+      </c>
+      <c r="F31" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G31" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H31" s="2">
+        <f t="shared" si="46"/>
+        <v>1</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A32" s="1">
+        <v>23</v>
+      </c>
+      <c r="B32" s="1">
+        <v>59</v>
+      </c>
+      <c r="C32" s="1">
+        <v>59</v>
+      </c>
+      <c r="D32" s="7">
+        <f t="shared" si="42"/>
+        <v>0.99998842592592596</v>
+      </c>
+      <c r="E32" s="9">
+        <f t="shared" si="43"/>
+        <v>0.99998842592592596</v>
+      </c>
+      <c r="F32" s="2">
+        <f t="shared" si="44"/>
+        <v>23</v>
+      </c>
+      <c r="G32" s="2">
+        <f t="shared" si="45"/>
+        <v>59</v>
+      </c>
+      <c r="H32" s="2">
+        <f t="shared" si="46"/>
+        <v>59</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A33" s="1">
+        <v>23</v>
+      </c>
+      <c r="B33" s="1">
+        <v>59</v>
+      </c>
+      <c r="C33" s="1">
+        <v>60</v>
+      </c>
+      <c r="D33" s="7">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="E33" s="9">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="F33" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G33" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H33" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A34" s="1">
+        <v>0</v>
+      </c>
+      <c r="B34" s="1">
+        <v>0</v>
+      </c>
+      <c r="C34" s="1">
+        <v>86399</v>
+      </c>
+      <c r="D34" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E34" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F34" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G34" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H34" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="1">
+        <v>0</v>
+      </c>
+      <c r="B35" s="1">
+        <v>0</v>
+      </c>
+      <c r="C35" s="1">
+        <v>86400</v>
+      </c>
+      <c r="D35" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E35" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F35" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G35" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H35" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="1">
+        <v>0</v>
+      </c>
+      <c r="B36" s="1">
+        <v>0</v>
+      </c>
+      <c r="C36" s="1">
+        <v>86401</v>
+      </c>
+      <c r="D36" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E36" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F36" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G36" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H36" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="1">
+        <v>0</v>
+      </c>
+      <c r="B37" s="1">
+        <v>1440</v>
+      </c>
+      <c r="C37" s="1">
+        <v>0</v>
+      </c>
+      <c r="D37" s="7">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="E37" s="9">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="F37" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G37" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H37" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="1">
+        <v>24</v>
+      </c>
+      <c r="B38" s="1">
+        <v>0</v>
+      </c>
+      <c r="C38" s="1">
+        <v>0</v>
+      </c>
+      <c r="D38" s="7">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="E38" s="9">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="F38" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G38" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H38" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="1">
+        <v>48</v>
+      </c>
+      <c r="B39" s="1">
+        <v>0</v>
+      </c>
+      <c r="C39" s="1">
+        <v>0</v>
+      </c>
+      <c r="D39" s="7">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="E39" s="9">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="F39" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G39" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H39" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="1">
+        <v>-1</v>
+      </c>
+      <c r="B40" s="1">
+        <v>-1</v>
+      </c>
+      <c r="C40" s="1">
+        <v>-1</v>
+      </c>
+      <c r="D40" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E40" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F40" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G40" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H40" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="11">
+        <v>-9.9999999999999995E-8</v>
+      </c>
+      <c r="B41" s="11">
+        <v>-9.9999999999999995E-8</v>
+      </c>
+      <c r="C41" s="11">
+        <v>-9.9999999999999995E-8</v>
+      </c>
+      <c r="D41" s="7">
+        <f t="shared" ref="D41" si="47">TIME(A41,B41,C41)</f>
+        <v>0</v>
+      </c>
+      <c r="E41" s="9">
+        <f t="shared" ref="E41" si="48">D41</f>
+        <v>0</v>
+      </c>
+      <c r="F41" s="2">
+        <f t="shared" ref="F41" si="49">HOUR(D41)</f>
+        <v>0</v>
+      </c>
+      <c r="G41" s="2">
+        <f t="shared" ref="G41" si="50">MINUTE(D41)</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="2">
+        <f t="shared" ref="H41" si="51">SECOND(D41)</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="1">
+        <v>0</v>
+      </c>
+      <c r="B42" s="1">
+        <v>0</v>
+      </c>
+      <c r="C42" s="1">
+        <v>-1</v>
+      </c>
+      <c r="D42" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E42" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F42" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G42" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H42" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="1">
+        <v>0</v>
+      </c>
+      <c r="B43" s="1">
+        <v>-1</v>
+      </c>
+      <c r="C43" s="1">
+        <v>0</v>
+      </c>
+      <c r="D43" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E43" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F43" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G43" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H43" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="1">
+        <v>1</v>
+      </c>
+      <c r="B44" s="1">
+        <v>1</v>
+      </c>
+      <c r="C44" s="1">
+        <v>0.49990000000000001</v>
+      </c>
+      <c r="D44" s="7">
+        <f t="shared" si="42"/>
+        <v>4.2361111111111113E-2</v>
+      </c>
+      <c r="E44" s="9">
+        <f t="shared" si="43"/>
+        <v>4.2361111111111113E-2</v>
+      </c>
+      <c r="F44" s="2">
+        <f t="shared" si="44"/>
+        <v>1</v>
+      </c>
+      <c r="G44" s="2">
+        <f t="shared" si="45"/>
+        <v>1</v>
+      </c>
+      <c r="H44" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="1">
+        <v>1</v>
+      </c>
+      <c r="B45" s="1">
+        <v>1</v>
+      </c>
+      <c r="C45" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="D45" s="7">
+        <f t="shared" si="42"/>
+        <v>4.2361111111111113E-2</v>
+      </c>
+      <c r="E45" s="9">
+        <f t="shared" si="43"/>
+        <v>4.2361111111111113E-2</v>
+      </c>
+      <c r="F45" s="2">
+        <f t="shared" si="44"/>
+        <v>1</v>
+      </c>
+      <c r="G45" s="2">
+        <f t="shared" si="45"/>
+        <v>1</v>
+      </c>
+      <c r="H45" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="1">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="B46" s="1">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="C46" s="1">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="D46" s="7">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="E46" s="9">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="F46" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G46" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H46" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E48" s="1">
+        <f>DATE(2025,6,15)+TIME(14,30,45)</f>
+        <v>45823.604687500003</v>
+      </c>
+      <c r="F48" s="2">
+        <f t="shared" ref="F48:F61" si="52">HOUR(E48)</f>
+        <v>14</v>
+      </c>
+      <c r="G48" s="2">
+        <f t="shared" ref="G48:G61" si="53">MINUTE(E48)</f>
+        <v>30</v>
+      </c>
+      <c r="H48" s="2">
+        <f t="shared" ref="H48:H61" si="54">SECOND(E48)</f>
+        <v>45</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="49" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E49" s="1">
+        <f>DATE(2025,6,15)</f>
+        <v>45823</v>
+      </c>
+      <c r="F49" s="2">
+        <f t="shared" si="52"/>
+        <v>0</v>
+      </c>
+      <c r="G49" s="2">
+        <f t="shared" si="53"/>
+        <v>0</v>
+      </c>
+      <c r="H49" s="2">
+        <f t="shared" si="54"/>
+        <v>0</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="50" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E50" s="1">
+        <v>0</v>
+      </c>
+      <c r="F50" s="2">
+        <f t="shared" si="52"/>
+        <v>0</v>
+      </c>
+      <c r="G50" s="2">
+        <f t="shared" si="53"/>
+        <v>0</v>
+      </c>
+      <c r="H50" s="2">
+        <f t="shared" si="54"/>
+        <v>0</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="51" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E51" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="F51" s="2">
+        <f t="shared" si="52"/>
+        <v>12</v>
+      </c>
+      <c r="G51" s="2">
+        <f t="shared" si="53"/>
+        <v>0</v>
+      </c>
+      <c r="H51" s="2">
+        <f t="shared" si="54"/>
+        <v>0</v>
+      </c>
+      <c r="I51" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="52" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E52" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="F52" s="2">
+        <f t="shared" si="52"/>
+        <v>6</v>
+      </c>
+      <c r="G52" s="2">
+        <f t="shared" si="53"/>
+        <v>0</v>
+      </c>
+      <c r="H52" s="2">
+        <f t="shared" si="54"/>
+        <v>0</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="53" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E53" s="1">
+        <v>1.0000000010000001</v>
+      </c>
+      <c r="F53" s="2">
+        <f t="shared" si="52"/>
+        <v>0</v>
+      </c>
+      <c r="G53" s="2">
+        <f t="shared" si="53"/>
+        <v>0</v>
+      </c>
+      <c r="H53" s="2">
+        <f t="shared" si="54"/>
+        <v>0</v>
+      </c>
+      <c r="I53" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="54" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E54" s="1">
+        <v>1</v>
+      </c>
+      <c r="F54" s="2">
+        <f t="shared" si="52"/>
+        <v>0</v>
+      </c>
+      <c r="G54" s="2">
+        <f t="shared" si="53"/>
+        <v>0</v>
+      </c>
+      <c r="H54" s="2">
+        <f t="shared" si="54"/>
+        <v>0</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="55" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E55" s="1">
+        <v>-0.5</v>
+      </c>
+      <c r="F55" s="2" t="e">
+        <f t="shared" si="52"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G55" s="2" t="e">
+        <f t="shared" si="53"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H55" s="2" t="e">
+        <f t="shared" si="54"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="56" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E56" s="1">
+        <v>-1</v>
+      </c>
+      <c r="F56" s="2" t="e">
+        <f t="shared" si="52"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G56" s="2" t="e">
+        <f t="shared" si="53"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H56" s="2" t="e">
+        <f t="shared" si="54"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="57" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E57" s="11">
+        <v>-9.9999999999999995E-8</v>
+      </c>
+      <c r="F57" s="2" t="e">
+        <f t="shared" ref="F57" si="55">HOUR(E57)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="G57" s="2" t="e">
+        <f t="shared" ref="G57" si="56">MINUTE(E57)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="H57" s="2" t="e">
+        <f t="shared" ref="H57" si="57">SECOND(E57)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="I57" s="10" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="58" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E58" s="1">
+        <f>DATE(9999,12,31)+0.9999999</f>
+        <v>2958465.9999998999</v>
+      </c>
+      <c r="F58" s="2" t="e">
+        <f t="shared" si="52"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G58" s="2" t="e">
+        <f t="shared" si="53"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H58" s="2" t="e">
+        <f t="shared" si="54"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="59" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E59" s="1">
+        <v>2958466</v>
+      </c>
+      <c r="F59" s="2" t="e">
+        <f t="shared" si="52"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G59" s="2" t="e">
+        <f t="shared" si="53"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H59" s="2" t="e">
+        <f t="shared" si="54"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="60" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E60" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F60" s="2">
+        <f t="shared" si="52"/>
+        <v>0</v>
+      </c>
+      <c r="G60" s="2">
+        <f t="shared" si="53"/>
+        <v>0</v>
+      </c>
+      <c r="H60" s="2">
+        <f t="shared" si="54"/>
+        <v>0</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="61" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E61" s="1" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="C22" s="1">
-        <v>3</v>
-      </c>
-      <c r="D22" s="7" t="e">
-        <f t="shared" si="29"/>
+      <c r="F61" s="2" t="e">
+        <f t="shared" si="52"/>
         <v>#N/A</v>
       </c>
-      <c r="E22" s="4" t="e">
-        <f t="shared" si="1"/>
+      <c r="G61" s="2" t="e">
+        <f t="shared" si="53"/>
         <v>#N/A</v>
       </c>
-      <c r="F22" s="2" t="e">
-        <f t="shared" si="30"/>
+      <c r="H61" s="2" t="e">
+        <f t="shared" si="54"/>
         <v>#N/A</v>
       </c>
-      <c r="G22" s="2" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H22" s="2" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I22" s="1" t="s">
+      <c r="I61" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
-      <c r="A23" s="1">
-        <v>1</v>
-      </c>
-      <c r="B23" s="1">
-        <v>2</v>
-      </c>
-      <c r="C23" s="1" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D23" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="E23" s="4" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="F23" s="2" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="G23" s="2" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H23" s="2" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D24" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E24" s="4" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F24" s="2" t="e">
-        <f t="shared" ref="F24" si="33">HOUR(D24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G24" s="2" t="e">
-        <f t="shared" ref="G24" si="34">MINUTE(D24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H24" s="2" t="e">
-        <f t="shared" ref="H24" si="35">SECOND(D24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D25" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E25" s="4" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F25" s="2" t="e">
-        <f t="shared" ref="F25" si="36">HOUR(D25)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G25" s="2" t="e">
-        <f t="shared" ref="G25" si="37">MINUTE(D25)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H25" s="2" t="e">
-        <f t="shared" ref="H25" si="38">SECOND(D25)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="A26" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="B26" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="D26" s="7">
-        <f t="shared" si="29"/>
-        <v>4.1678240740740738E-2</v>
-      </c>
-      <c r="E26" s="4">
-        <f t="shared" si="1"/>
-        <v>4.1678240740740738E-2</v>
-      </c>
-      <c r="F26" s="2">
-        <f t="shared" ref="F26" si="39">HOUR(D26)</f>
-        <v>1</v>
-      </c>
-      <c r="G26" s="2">
-        <f t="shared" ref="G26" si="40">MINUTE(D26)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="2">
-        <f t="shared" ref="H26" si="41">SECOND(D26)</f>
-        <v>1</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9"/>
-    <row r="28" spans="1:9"/>
-    <row r="29" spans="1:9"/>
-    <row r="30" spans="1:9"/>
-    <row r="31" spans="1:9"/>
-    <row r="32" spans="1:9"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update: add xlsx tests for TIME, HOUR, MINUTE, SECOND
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/DATE_AND_TIME/TIME_HOUR_MINUTE_SECOND.xlsx
+++ b/xlsx/tests/calc_tests/DATE_AND_TIME/TIME_HOUR_MINUTE_SECOND.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elsam\Documents\IronCalc stuff\my_calc_tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A35D429E-2E32-4024-9948-77450FEAF236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC13EEDE-8837-4993-87AA-6A70A628400A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5990" yWindow="3860" windowWidth="28800" windowHeight="15290" xr2:uid="{F5EF1803-C89D-8542-8C3F-E05EFF447D52}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{F5EF1803-C89D-8542-8C3F-E05EFF447D52}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="50">
   <si>
     <t>HOUR</t>
   </si>
@@ -135,18 +135,6 @@
     <t>Boolean as input</t>
   </si>
   <si>
-    <t>Hours beyond the 32767 bound</t>
-  </si>
-  <si>
-    <t>Minutes beyond the 32767 bound</t>
-  </si>
-  <si>
-    <t>Seconds beyond the 32767 bound</t>
-  </si>
-  <si>
-    <t>One argument beyond bound, others at bound</t>
-  </si>
-  <si>
     <t>All arguments zero</t>
   </si>
   <si>
@@ -159,15 +147,6 @@
     <t>Seconds roll over into the next day</t>
   </si>
   <si>
-    <t>Seconds equal to one day minus one</t>
-  </si>
-  <si>
-    <t>Seconds equal to exactly one day</t>
-  </si>
-  <si>
-    <t>Seconds just beyond one day</t>
-  </si>
-  <si>
     <t>Minutes equal to exactly one day</t>
   </si>
   <si>
@@ -219,12 +198,6 @@
     <t>Negative whole serial</t>
   </si>
   <si>
-    <t>Maximum date with a time portion</t>
-  </si>
-  <si>
-    <t>Serial beyond the maximum date</t>
-  </si>
-  <si>
     <t>Serial just above one whole day</t>
   </si>
   <si>
@@ -235,9 +208,6 @@
   </si>
   <si>
     <t>Negative near zero</t>
-  </si>
-  <si>
-    <t>All arguments negative near zero</t>
   </si>
 </sst>
 </file>
@@ -357,6 +327,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFEDDAB1"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -707,8 +682,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4323771-C859-F046-B681-A08AFC84A35B}">
-  <dimension ref="A1:I61"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I51"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12.25" style="1" customWidth="1"/>
     <col min="2" max="3" width="11" style="1"/>
@@ -719,7 +694,7 @@
     <col min="10" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -745,7 +720,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>3</v>
       </c>
@@ -776,7 +751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A3" s="1">
         <v>24</v>
       </c>
@@ -810,7 +785,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A4" s="1">
         <v>16</v>
       </c>
@@ -844,7 +819,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A5" s="1">
         <v>3.1</v>
       </c>
@@ -878,7 +853,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A6" s="1">
         <v>23</v>
       </c>
@@ -912,7 +887,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="D7" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -937,7 +912,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>23</v>
       </c>
@@ -965,7 +940,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="B9" s="1">
         <v>23</v>
       </c>
@@ -993,7 +968,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="C10" s="1">
         <v>23</v>
       </c>
@@ -1021,7 +996,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>-1</v>
       </c>
@@ -1055,7 +1030,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <v>12</v>
       </c>
@@ -1089,7 +1064,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <v>13</v>
       </c>
@@ -1123,7 +1098,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <v>34</v>
       </c>
@@ -1157,7 +1132,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
         <v>10</v>
       </c>
@@ -1191,7 +1166,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
         <v>10</v>
       </c>
@@ -1225,7 +1200,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
         <v>32767</v>
       </c>
@@ -1259,7 +1234,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
@@ -1294,7 +1269,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
         <v>1</v>
       </c>
@@ -1314,22 +1289,22 @@
         <v>#DIV/0!</v>
       </c>
       <c r="F19" s="2" t="e">
-        <f t="shared" ref="F19:F21" si="30">HOUR(D19)</f>
+        <f t="shared" ref="F19:F20" si="30">HOUR(D19)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G19" s="2" t="e">
-        <f t="shared" ref="G19:G21" si="31">MINUTE(D19)</f>
+        <f t="shared" ref="G19:G20" si="31">MINUTE(D19)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="H19" s="2" t="e">
-        <f t="shared" ref="H19:H21" si="32">SECOND(D19)</f>
+        <f t="shared" ref="H19:H20" si="32">SECOND(D19)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
         <v>1</v>
       </c>
@@ -1364,7 +1339,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="e">
         <f>NA()</f>
         <v>#N/A</v>
@@ -1378,30 +1353,30 @@
         <v>#NAME?</v>
       </c>
       <c r="D21" s="7" t="e">
-        <f t="shared" ca="1" si="29"/>
+        <f ca="1">TIME(A21,B21,C21)</f>
         <v>#N/A</v>
       </c>
       <c r="E21" s="4" t="e">
-        <f t="shared" ca="1" si="1"/>
+        <f ca="1">D21</f>
         <v>#N/A</v>
       </c>
       <c r="F21" s="2" t="e">
-        <f t="shared" ca="1" si="30"/>
+        <f ca="1">HOUR(D21)</f>
         <v>#N/A</v>
       </c>
       <c r="G21" s="2" t="e">
-        <f t="shared" ca="1" si="31"/>
+        <f ca="1">MINUTE(D21)</f>
         <v>#N/A</v>
       </c>
       <c r="H21" s="2" t="e">
-        <f t="shared" ca="1" si="32"/>
+        <f ca="1">SECOND(D21)</f>
         <v>#N/A</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A22" s="1" t="s">
         <v>17</v>
       </c>
@@ -1435,7 +1410,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -1469,7 +1444,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A24" s="1" t="b">
         <v>1</v>
       </c>
@@ -1503,280 +1478,280 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="14.5" x14ac:dyDescent="0.35"/>
-    <row r="26" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" ht="14.25" x14ac:dyDescent="0.45"/>
+    <row r="26" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A26" s="1">
-        <v>32768</v>
+        <v>0</v>
       </c>
       <c r="B26" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C26" s="1">
-        <v>1</v>
-      </c>
-      <c r="D26" s="7" t="e">
-        <f t="shared" ref="D26:D46" si="42">TIME(A26,B26,C26)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="E26" s="9" t="e">
-        <f t="shared" ref="E26:E46" si="43">D26</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="F26" s="2" t="e">
-        <f t="shared" ref="F26:F46" si="44">HOUR(D26)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="G26" s="2" t="e">
-        <f t="shared" ref="G26:G46" si="45">MINUTE(D26)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="H26" s="2" t="e">
-        <f t="shared" ref="H26:H46" si="46">SECOND(D26)</f>
-        <v>#NUM!</v>
+        <v>0</v>
+      </c>
+      <c r="D26" s="7">
+        <f>TIME(A26,B26,C26)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="9">
+        <f>D26</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="2">
+        <f>HOUR(D26)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="2">
+        <f>MINUTE(D26)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="2">
+        <f>SECOND(D26)</f>
+        <v>0</v>
       </c>
       <c r="I26" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A27" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B27" s="1">
-        <v>32768</v>
+        <v>0</v>
       </c>
       <c r="C27" s="1">
         <v>1</v>
       </c>
-      <c r="D27" s="7" t="e">
-        <f t="shared" si="42"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="E27" s="9" t="e">
-        <f t="shared" si="43"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="F27" s="2" t="e">
-        <f t="shared" si="44"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="G27" s="2" t="e">
-        <f t="shared" si="45"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="H27" s="2" t="e">
-        <f t="shared" si="46"/>
-        <v>#NUM!</v>
+      <c r="D27" s="7">
+        <f>TIME(A27,B27,C27)</f>
+        <v>1.1574074074074073E-5</v>
+      </c>
+      <c r="E27" s="9">
+        <f>D27</f>
+        <v>1.1574074074074073E-5</v>
+      </c>
+      <c r="F27" s="2">
+        <f>HOUR(D27)</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="2">
+        <f>MINUTE(D27)</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="2">
+        <f>SECOND(D27)</f>
+        <v>1</v>
       </c>
       <c r="I27" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A28" s="1">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="B28" s="1">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="C28" s="1">
-        <v>32768</v>
-      </c>
-      <c r="D28" s="7" t="e">
-        <f t="shared" si="42"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="E28" s="9" t="e">
-        <f t="shared" si="43"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="F28" s="2" t="e">
-        <f t="shared" si="44"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="G28" s="2" t="e">
-        <f t="shared" si="45"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="H28" s="2" t="e">
-        <f t="shared" si="46"/>
-        <v>#NUM!</v>
+        <v>59</v>
+      </c>
+      <c r="D28" s="7">
+        <f>TIME(A28,B28,C28)</f>
+        <v>0.99998842592592596</v>
+      </c>
+      <c r="E28" s="9">
+        <f>D28</f>
+        <v>0.99998842592592596</v>
+      </c>
+      <c r="F28" s="2">
+        <f>HOUR(D28)</f>
+        <v>23</v>
+      </c>
+      <c r="G28" s="2">
+        <f>MINUTE(D28)</f>
+        <v>59</v>
+      </c>
+      <c r="H28" s="2">
+        <f>SECOND(D28)</f>
+        <v>59</v>
       </c>
       <c r="I28" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A29" s="1">
-        <v>32767</v>
+        <v>23</v>
       </c>
       <c r="B29" s="1">
-        <v>32767</v>
+        <v>59</v>
       </c>
       <c r="C29" s="1">
-        <v>32768</v>
-      </c>
-      <c r="D29" s="7" t="e">
-        <f t="shared" si="42"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="E29" s="9" t="e">
-        <f t="shared" si="43"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="F29" s="2" t="e">
-        <f t="shared" si="44"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="G29" s="2" t="e">
-        <f t="shared" si="45"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="H29" s="2" t="e">
-        <f t="shared" si="46"/>
-        <v>#NUM!</v>
+        <v>60</v>
+      </c>
+      <c r="D29" s="7">
+        <f>TIME(A29,B29,C29)</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="9">
+        <f>D29</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="2">
+        <f>HOUR(D29)</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="2">
+        <f>MINUTE(D29)</f>
+        <v>0</v>
+      </c>
+      <c r="H29" s="2">
+        <f>SECOND(D29)</f>
+        <v>0</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="1">
         <v>0</v>
       </c>
       <c r="B30" s="1">
-        <v>0</v>
+        <v>1440</v>
       </c>
       <c r="C30" s="1">
         <v>0</v>
       </c>
       <c r="D30" s="7">
-        <f t="shared" si="42"/>
+        <f>TIME(A30,B30,C30)</f>
         <v>0</v>
       </c>
       <c r="E30" s="9">
-        <f t="shared" si="43"/>
+        <f>D30</f>
         <v>0</v>
       </c>
       <c r="F30" s="2">
-        <f t="shared" si="44"/>
+        <f>HOUR(D30)</f>
         <v>0</v>
       </c>
       <c r="G30" s="2">
-        <f t="shared" si="45"/>
+        <f>MINUTE(D30)</f>
         <v>0</v>
       </c>
       <c r="H30" s="2">
-        <f t="shared" si="46"/>
+        <f>SECOND(D30)</f>
         <v>0</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="1">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="B31" s="1">
         <v>0</v>
       </c>
       <c r="C31" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" s="7">
-        <f t="shared" si="42"/>
-        <v>1.1574074074074073E-5</v>
+        <f>TIME(A31,B31,C31)</f>
+        <v>0</v>
       </c>
       <c r="E31" s="9">
-        <f t="shared" si="43"/>
-        <v>1.1574074074074073E-5</v>
+        <f>D31</f>
+        <v>0</v>
       </c>
       <c r="F31" s="2">
-        <f t="shared" si="44"/>
+        <f>HOUR(D31)</f>
         <v>0</v>
       </c>
       <c r="G31" s="2">
-        <f t="shared" si="45"/>
+        <f>MINUTE(D31)</f>
         <v>0</v>
       </c>
       <c r="H31" s="2">
-        <f t="shared" si="46"/>
-        <v>1</v>
+        <f>SECOND(D31)</f>
+        <v>0</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="1">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="B32" s="1">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="C32" s="1">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="D32" s="7">
-        <f t="shared" si="42"/>
-        <v>0.99998842592592596</v>
+        <f>TIME(A32,B32,C32)</f>
+        <v>0</v>
       </c>
       <c r="E32" s="9">
-        <f t="shared" si="43"/>
-        <v>0.99998842592592596</v>
+        <f>D32</f>
+        <v>0</v>
       </c>
       <c r="F32" s="2">
-        <f t="shared" si="44"/>
-        <v>23</v>
+        <f>HOUR(D32)</f>
+        <v>0</v>
       </c>
       <c r="G32" s="2">
-        <f t="shared" si="45"/>
-        <v>59</v>
+        <f>MINUTE(D32)</f>
+        <v>0</v>
       </c>
       <c r="H32" s="2">
-        <f t="shared" si="46"/>
-        <v>59</v>
+        <f>SECOND(D32)</f>
+        <v>0</v>
       </c>
       <c r="I32" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="1">
-        <v>23</v>
+        <v>-1</v>
       </c>
       <c r="B33" s="1">
-        <v>59</v>
+        <v>-1</v>
       </c>
       <c r="C33" s="1">
-        <v>60</v>
-      </c>
-      <c r="D33" s="7">
-        <f t="shared" si="42"/>
-        <v>0</v>
-      </c>
-      <c r="E33" s="9">
-        <f t="shared" si="43"/>
-        <v>0</v>
-      </c>
-      <c r="F33" s="2">
-        <f t="shared" si="44"/>
-        <v>0</v>
-      </c>
-      <c r="G33" s="2">
-        <f t="shared" si="45"/>
-        <v>0</v>
-      </c>
-      <c r="H33" s="2">
-        <f t="shared" si="46"/>
-        <v>0</v>
+        <v>-1</v>
+      </c>
+      <c r="D33" s="7" t="e">
+        <f>TIME(A33,B33,C33)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="E33" s="9" t="e">
+        <f>D33</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="F33" s="2" t="e">
+        <f>HOUR(D33)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="G33" s="2" t="e">
+        <f>MINUTE(D33)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="H33" s="2" t="e">
+        <f>SECOND(D33)</f>
+        <v>#NUM!</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="1">
         <v>0</v>
       </c>
@@ -1784,721 +1759,408 @@
         <v>0</v>
       </c>
       <c r="C34" s="1">
-        <v>86399</v>
+        <v>-1</v>
       </c>
       <c r="D34" s="7" t="e">
-        <f t="shared" si="42"/>
+        <f>TIME(A34,B34,C34)</f>
         <v>#NUM!</v>
       </c>
       <c r="E34" s="9" t="e">
-        <f t="shared" si="43"/>
+        <f>D34</f>
         <v>#NUM!</v>
       </c>
       <c r="F34" s="2" t="e">
-        <f t="shared" si="44"/>
+        <f>HOUR(D34)</f>
         <v>#NUM!</v>
       </c>
       <c r="G34" s="2" t="e">
-        <f t="shared" si="45"/>
+        <f>MINUTE(D34)</f>
         <v>#NUM!</v>
       </c>
       <c r="H34" s="2" t="e">
-        <f t="shared" si="46"/>
+        <f>SECOND(D34)</f>
         <v>#NUM!</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="1">
         <v>0</v>
       </c>
       <c r="B35" s="1">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="C35" s="1">
-        <v>86400</v>
+        <v>0</v>
       </c>
       <c r="D35" s="7" t="e">
-        <f t="shared" si="42"/>
+        <f>TIME(A35,B35,C35)</f>
         <v>#NUM!</v>
       </c>
       <c r="E35" s="9" t="e">
-        <f t="shared" si="43"/>
+        <f>D35</f>
         <v>#NUM!</v>
       </c>
       <c r="F35" s="2" t="e">
-        <f t="shared" si="44"/>
+        <f>HOUR(D35)</f>
         <v>#NUM!</v>
       </c>
       <c r="G35" s="2" t="e">
-        <f t="shared" si="45"/>
+        <f>MINUTE(D35)</f>
         <v>#NUM!</v>
       </c>
       <c r="H35" s="2" t="e">
-        <f t="shared" si="46"/>
+        <f>SECOND(D35)</f>
         <v>#NUM!</v>
       </c>
       <c r="I35" s="1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B36" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C36" s="1">
-        <v>86401</v>
-      </c>
-      <c r="D36" s="7" t="e">
-        <f t="shared" si="42"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="E36" s="9" t="e">
-        <f t="shared" si="43"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="F36" s="2" t="e">
-        <f t="shared" si="44"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="G36" s="2" t="e">
-        <f t="shared" si="45"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="H36" s="2" t="e">
-        <f t="shared" si="46"/>
-        <v>#NUM!</v>
+        <v>0.49990000000000001</v>
+      </c>
+      <c r="D36" s="7">
+        <f>TIME(A36,B36,C36)</f>
+        <v>4.2361111111111113E-2</v>
+      </c>
+      <c r="E36" s="9">
+        <f>D36</f>
+        <v>4.2361111111111113E-2</v>
+      </c>
+      <c r="F36" s="2">
+        <f>HOUR(D36)</f>
+        <v>1</v>
+      </c>
+      <c r="G36" s="2">
+        <f>MINUTE(D36)</f>
+        <v>1</v>
+      </c>
+      <c r="H36" s="2">
+        <f>SECOND(D36)</f>
+        <v>0</v>
       </c>
       <c r="I36" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B37" s="1">
-        <v>1440</v>
+        <v>1</v>
       </c>
       <c r="C37" s="1">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D37" s="7">
-        <f t="shared" si="42"/>
-        <v>0</v>
+        <f>TIME(A37,B37,C37)</f>
+        <v>4.2361111111111113E-2</v>
       </c>
       <c r="E37" s="9">
-        <f t="shared" si="43"/>
-        <v>0</v>
+        <f>D37</f>
+        <v>4.2361111111111113E-2</v>
       </c>
       <c r="F37" s="2">
-        <f t="shared" si="44"/>
-        <v>0</v>
+        <f>HOUR(D37)</f>
+        <v>1</v>
       </c>
       <c r="G37" s="2">
-        <f t="shared" si="45"/>
-        <v>0</v>
+        <f>MINUTE(D37)</f>
+        <v>1</v>
       </c>
       <c r="H37" s="2">
-        <f t="shared" si="46"/>
+        <f>SECOND(D37)</f>
         <v>0</v>
       </c>
       <c r="I37" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="1">
-        <v>24</v>
+        <v>1.0000000000000001E-9</v>
       </c>
       <c r="B38" s="1">
-        <v>0</v>
+        <v>1.0000000000000001E-9</v>
       </c>
       <c r="C38" s="1">
-        <v>0</v>
+        <v>1.0000000000000001E-9</v>
       </c>
       <c r="D38" s="7">
-        <f t="shared" si="42"/>
+        <f>TIME(A38,B38,C38)</f>
         <v>0</v>
       </c>
       <c r="E38" s="9">
-        <f t="shared" si="43"/>
+        <f>D38</f>
         <v>0</v>
       </c>
       <c r="F38" s="2">
-        <f t="shared" si="44"/>
+        <f>HOUR(D38)</f>
         <v>0</v>
       </c>
       <c r="G38" s="2">
-        <f t="shared" si="45"/>
+        <f>MINUTE(D38)</f>
         <v>0</v>
       </c>
       <c r="H38" s="2">
-        <f t="shared" si="46"/>
+        <f>SECOND(D38)</f>
         <v>0</v>
       </c>
       <c r="I38" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="1">
-        <v>48</v>
-      </c>
-      <c r="B39" s="1">
-        <v>0</v>
-      </c>
-      <c r="C39" s="1">
-        <v>0</v>
-      </c>
-      <c r="D39" s="7">
+    <row r="40" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E40" s="1">
+        <f>DATE(2025,6,15)+TIME(14,30,45)</f>
+        <v>45823.604687500003</v>
+      </c>
+      <c r="F40" s="2">
+        <f t="shared" ref="F40:F51" si="42">HOUR(E40)</f>
+        <v>14</v>
+      </c>
+      <c r="G40" s="2">
+        <f t="shared" ref="G40:G51" si="43">MINUTE(E40)</f>
+        <v>30</v>
+      </c>
+      <c r="H40" s="2">
+        <f t="shared" ref="H40:H51" si="44">SECOND(E40)</f>
+        <v>45</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E41" s="1">
+        <f>DATE(2025,6,15)</f>
+        <v>45823</v>
+      </c>
+      <c r="F41" s="2">
         <f t="shared" si="42"/>
         <v>0</v>
       </c>
-      <c r="E39" s="9">
+      <c r="G41" s="2">
         <f t="shared" si="43"/>
         <v>0</v>
       </c>
-      <c r="F39" s="2">
+      <c r="H41" s="2">
         <f t="shared" si="44"/>
         <v>0</v>
       </c>
-      <c r="G39" s="2">
-        <f t="shared" si="45"/>
-        <v>0</v>
-      </c>
-      <c r="H39" s="2">
-        <f t="shared" si="46"/>
-        <v>0</v>
-      </c>
-      <c r="I39" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="1">
-        <v>-1</v>
-      </c>
-      <c r="B40" s="1">
-        <v>-1</v>
-      </c>
-      <c r="C40" s="1">
-        <v>-1</v>
-      </c>
-      <c r="D40" s="7" t="e">
+      <c r="I41" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E42" s="1">
+        <v>0</v>
+      </c>
+      <c r="F42" s="2">
         <f t="shared" si="42"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="E40" s="9" t="e">
+        <v>0</v>
+      </c>
+      <c r="G42" s="2">
         <f t="shared" si="43"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="F40" s="2" t="e">
+        <v>0</v>
+      </c>
+      <c r="H42" s="2">
         <f t="shared" si="44"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="G40" s="2" t="e">
-        <f t="shared" si="45"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="H40" s="2" t="e">
-        <f t="shared" si="46"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="I40" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="11">
-        <v>-9.9999999999999995E-8</v>
-      </c>
-      <c r="B41" s="11">
-        <v>-9.9999999999999995E-8</v>
-      </c>
-      <c r="C41" s="11">
-        <v>-9.9999999999999995E-8</v>
-      </c>
-      <c r="D41" s="7">
-        <f t="shared" ref="D41" si="47">TIME(A41,B41,C41)</f>
-        <v>0</v>
-      </c>
-      <c r="E41" s="9">
-        <f t="shared" ref="E41" si="48">D41</f>
-        <v>0</v>
-      </c>
-      <c r="F41" s="2">
-        <f t="shared" ref="F41" si="49">HOUR(D41)</f>
-        <v>0</v>
-      </c>
-      <c r="G41" s="2">
-        <f t="shared" ref="G41" si="50">MINUTE(D41)</f>
-        <v>0</v>
-      </c>
-      <c r="H41" s="2">
-        <f t="shared" ref="H41" si="51">SECOND(D41)</f>
-        <v>0</v>
-      </c>
-      <c r="I41" s="10" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="1">
-        <v>0</v>
-      </c>
-      <c r="B42" s="1">
-        <v>0</v>
-      </c>
-      <c r="C42" s="1">
-        <v>-1</v>
-      </c>
-      <c r="D42" s="7" t="e">
-        <f t="shared" si="42"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="E42" s="9" t="e">
-        <f t="shared" si="43"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="F42" s="2" t="e">
-        <f t="shared" si="44"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="G42" s="2" t="e">
-        <f t="shared" si="45"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="H42" s="2" t="e">
-        <f t="shared" si="46"/>
-        <v>#NUM!</v>
+        <v>0</v>
       </c>
       <c r="I42" s="1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="1">
-        <v>0</v>
-      </c>
-      <c r="B43" s="1">
-        <v>-1</v>
-      </c>
-      <c r="C43" s="1">
-        <v>0</v>
-      </c>
-      <c r="D43" s="7" t="e">
+    <row r="43" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E43" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="F43" s="2">
         <f t="shared" si="42"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="E43" s="9" t="e">
+        <v>12</v>
+      </c>
+      <c r="G43" s="2">
         <f t="shared" si="43"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="F43" s="2" t="e">
+        <v>0</v>
+      </c>
+      <c r="H43" s="2">
         <f t="shared" si="44"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="G43" s="2" t="e">
-        <f t="shared" si="45"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="H43" s="2" t="e">
-        <f t="shared" si="46"/>
-        <v>#NUM!</v>
+        <v>0</v>
       </c>
       <c r="I43" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="1">
-        <v>1</v>
-      </c>
-      <c r="B44" s="1">
-        <v>1</v>
-      </c>
-      <c r="C44" s="1">
-        <v>0.49990000000000001</v>
-      </c>
-      <c r="D44" s="7">
+    <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E44" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="F44" s="2">
         <f t="shared" si="42"/>
-        <v>4.2361111111111113E-2</v>
-      </c>
-      <c r="E44" s="9">
+        <v>6</v>
+      </c>
+      <c r="G44" s="2">
         <f t="shared" si="43"/>
-        <v>4.2361111111111113E-2</v>
-      </c>
-      <c r="F44" s="2">
+        <v>0</v>
+      </c>
+      <c r="H44" s="2">
         <f t="shared" si="44"/>
-        <v>1</v>
-      </c>
-      <c r="G44" s="2">
-        <f t="shared" si="45"/>
-        <v>1</v>
-      </c>
-      <c r="H44" s="2">
-        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="I44" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="1">
-        <v>1</v>
-      </c>
-      <c r="B45" s="1">
-        <v>1</v>
-      </c>
-      <c r="C45" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="D45" s="7">
+    <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E45" s="1">
+        <v>1.0000000010000001</v>
+      </c>
+      <c r="F45" s="2">
         <f t="shared" si="42"/>
-        <v>4.2361111111111113E-2</v>
-      </c>
-      <c r="E45" s="9">
+        <v>0</v>
+      </c>
+      <c r="G45" s="2">
         <f t="shared" si="43"/>
-        <v>4.2361111111111113E-2</v>
-      </c>
-      <c r="F45" s="2">
+        <v>0</v>
+      </c>
+      <c r="H45" s="2">
         <f t="shared" si="44"/>
-        <v>1</v>
-      </c>
-      <c r="G45" s="2">
-        <f t="shared" si="45"/>
-        <v>1</v>
-      </c>
-      <c r="H45" s="2">
-        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="I45" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E46" s="1">
+        <v>1</v>
+      </c>
+      <c r="F46" s="2">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="G46" s="2">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="H46" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="I46" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="1">
-        <v>1.0000000000000001E-9</v>
-      </c>
-      <c r="B46" s="1">
-        <v>1.0000000000000001E-9</v>
-      </c>
-      <c r="C46" s="1">
-        <v>1.0000000000000001E-9</v>
-      </c>
-      <c r="D46" s="7">
+    <row r="47" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E47" s="1">
+        <v>-0.5</v>
+      </c>
+      <c r="F47" s="2" t="e">
         <f t="shared" si="42"/>
-        <v>0</v>
-      </c>
-      <c r="E46" s="9">
+        <v>#NUM!</v>
+      </c>
+      <c r="G47" s="2" t="e">
         <f t="shared" si="43"/>
-        <v>0</v>
-      </c>
-      <c r="F46" s="2">
+        <v>#NUM!</v>
+      </c>
+      <c r="H47" s="2" t="e">
         <f t="shared" si="44"/>
-        <v>0</v>
-      </c>
-      <c r="G46" s="2">
-        <f t="shared" si="45"/>
-        <v>0</v>
-      </c>
-      <c r="H46" s="2">
-        <f t="shared" si="46"/>
-        <v>0</v>
-      </c>
-      <c r="I46" s="1" t="s">
+        <v>#NUM!</v>
+      </c>
+      <c r="I47" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="E48" s="1">
-        <f>DATE(2025,6,15)+TIME(14,30,45)</f>
-        <v>45823.604687500003</v>
-      </c>
-      <c r="F48" s="2">
-        <f t="shared" ref="F48:F61" si="52">HOUR(E48)</f>
-        <v>14</v>
-      </c>
-      <c r="G48" s="2">
-        <f t="shared" ref="G48:G61" si="53">MINUTE(E48)</f>
-        <v>30</v>
-      </c>
-      <c r="H48" s="2">
-        <f t="shared" ref="H48:H61" si="54">SECOND(E48)</f>
-        <v>45</v>
+        <v>-1</v>
+      </c>
+      <c r="F48" s="2" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G48" s="2" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H48" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
       </c>
       <c r="I48" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="49" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E49" s="1">
-        <f>DATE(2025,6,15)</f>
-        <v>45823</v>
-      </c>
-      <c r="F49" s="2">
-        <f t="shared" si="52"/>
-        <v>0</v>
-      </c>
-      <c r="G49" s="2">
-        <f t="shared" si="53"/>
-        <v>0</v>
-      </c>
-      <c r="H49" s="2">
-        <f t="shared" si="54"/>
-        <v>0</v>
-      </c>
-      <c r="I49" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="50" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E50" s="1">
-        <v>0</v>
+    <row r="49" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E49" s="11">
+        <v>-9.9999999999999995E-8</v>
+      </c>
+      <c r="F49" s="2" t="e">
+        <f t="shared" ref="F49" si="45">HOUR(E49)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="G49" s="2" t="e">
+        <f t="shared" ref="G49" si="46">MINUTE(E49)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="H49" s="2" t="e">
+        <f t="shared" ref="H49" si="47">SECOND(E49)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="I49" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E50" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="F50" s="2">
-        <f t="shared" si="52"/>
+        <f t="shared" si="42"/>
         <v>0</v>
       </c>
       <c r="G50" s="2">
-        <f t="shared" si="53"/>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="H50" s="2">
-        <f t="shared" si="54"/>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="I50" s="1" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="51" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E51" s="1">
-        <v>0.5</v>
-      </c>
-      <c r="F51" s="2">
-        <f t="shared" si="52"/>
-        <v>12</v>
-      </c>
-      <c r="G51" s="2">
-        <f t="shared" si="53"/>
-        <v>0</v>
-      </c>
-      <c r="H51" s="2">
-        <f t="shared" si="54"/>
-        <v>0</v>
-      </c>
-      <c r="I51" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="52" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E52" s="1">
-        <v>0.25</v>
-      </c>
-      <c r="F52" s="2">
-        <f t="shared" si="52"/>
-        <v>6</v>
-      </c>
-      <c r="G52" s="2">
-        <f t="shared" si="53"/>
-        <v>0</v>
-      </c>
-      <c r="H52" s="2">
-        <f t="shared" si="54"/>
-        <v>0</v>
-      </c>
-      <c r="I52" s="1" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="53" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E53" s="1">
-        <v>1.0000000010000001</v>
-      </c>
-      <c r="F53" s="2">
-        <f t="shared" si="52"/>
-        <v>0</v>
-      </c>
-      <c r="G53" s="2">
-        <f t="shared" si="53"/>
-        <v>0</v>
-      </c>
-      <c r="H53" s="2">
-        <f t="shared" si="54"/>
-        <v>0</v>
-      </c>
-      <c r="I53" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="54" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E54" s="1">
-        <v>1</v>
-      </c>
-      <c r="F54" s="2">
-        <f t="shared" si="52"/>
-        <v>0</v>
-      </c>
-      <c r="G54" s="2">
-        <f t="shared" si="53"/>
-        <v>0</v>
-      </c>
-      <c r="H54" s="2">
-        <f t="shared" si="54"/>
-        <v>0</v>
-      </c>
-      <c r="I54" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="55" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E55" s="1">
-        <v>-0.5</v>
-      </c>
-      <c r="F55" s="2" t="e">
-        <f t="shared" si="52"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="G55" s="2" t="e">
-        <f t="shared" si="53"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="H55" s="2" t="e">
-        <f t="shared" si="54"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="I55" s="1" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="56" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E56" s="1">
-        <v>-1</v>
-      </c>
-      <c r="F56" s="2" t="e">
-        <f t="shared" si="52"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="G56" s="2" t="e">
-        <f t="shared" si="53"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="H56" s="2" t="e">
-        <f t="shared" si="54"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="I56" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="57" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E57" s="11">
-        <v>-9.9999999999999995E-8</v>
-      </c>
-      <c r="F57" s="2" t="e">
-        <f t="shared" ref="F57" si="55">HOUR(E57)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="G57" s="2" t="e">
-        <f t="shared" ref="G57" si="56">MINUTE(E57)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="H57" s="2" t="e">
-        <f t="shared" ref="H57" si="57">SECOND(E57)</f>
-        <v>#NUM!</v>
-      </c>
-      <c r="I57" s="10" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="58" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E58" s="1">
-        <f>DATE(9999,12,31)+0.9999999</f>
-        <v>2958465.9999998999</v>
-      </c>
-      <c r="F58" s="2" t="e">
-        <f t="shared" si="52"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="G58" s="2" t="e">
-        <f t="shared" si="53"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="H58" s="2" t="e">
-        <f t="shared" si="54"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="I58" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="59" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E59" s="1">
-        <v>2958466</v>
-      </c>
-      <c r="F59" s="2" t="e">
-        <f t="shared" si="52"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="G59" s="2" t="e">
-        <f t="shared" si="53"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="H59" s="2" t="e">
-        <f t="shared" si="54"/>
-        <v>#NUM!</v>
-      </c>
-      <c r="I59" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="60" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E60" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="F60" s="2">
-        <f t="shared" si="52"/>
-        <v>0</v>
-      </c>
-      <c r="G60" s="2">
-        <f t="shared" si="53"/>
-        <v>0</v>
-      </c>
-      <c r="H60" s="2">
-        <f t="shared" si="54"/>
-        <v>0</v>
-      </c>
-      <c r="I60" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="61" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="E61" s="1" t="e">
+    <row r="51" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E51" s="1" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="F61" s="2" t="e">
-        <f t="shared" si="52"/>
+      <c r="F51" s="2" t="e">
+        <f t="shared" si="42"/>
         <v>#N/A</v>
       </c>
-      <c r="G61" s="2" t="e">
-        <f t="shared" si="53"/>
+      <c r="G51" s="2" t="e">
+        <f t="shared" si="43"/>
         <v>#N/A</v>
       </c>
-      <c r="H61" s="2" t="e">
-        <f t="shared" si="54"/>
+      <c r="H51" s="2" t="e">
+        <f t="shared" si="44"/>
         <v>#N/A</v>
       </c>
-      <c r="I61" s="1" t="s">
+      <c r="I51" s="1" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update: add more test cases that cover #1432
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/DATE_AND_TIME/TIME_HOUR_MINUTE_SECOND.xlsx
+++ b/xlsx/tests/calc_tests/DATE_AND_TIME/TIME_HOUR_MINUTE_SECOND.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elsam\Documents\IronCalc stuff\my_calc_tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC13EEDE-8837-4993-87AA-6A70A628400A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC112A6F-ADF2-48B2-AF26-281DCF89B185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{F5EF1803-C89D-8542-8C3F-E05EFF447D52}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="57">
   <si>
     <t>HOUR</t>
   </si>
@@ -208,6 +208,27 @@
   </si>
   <si>
     <t>Negative near zero</t>
+  </si>
+  <si>
+    <t>Time 12:29:59.99997 as fractional</t>
+  </si>
+  <si>
+    <t>Time 0.4 ms under 12:30:00 rounds up: MINUTE 30, SECOND 0</t>
+  </si>
+  <si>
+    <t>Same as above with a date portion: MINUTE 30, SECOND 0</t>
+  </si>
+  <si>
+    <t>Arithmetic result just under 00:01:00: MINUTE 1, SECOND 0</t>
+  </si>
+  <si>
+    <t>Arithmetic result just under 3 s: MINUTE 0, SECOND 3</t>
+  </si>
+  <si>
+    <t>12:00:29.9996 rounds up to 30 s: MINUTE 0, SECOND 30</t>
+  </si>
+  <si>
+    <t>Existing behaviour kept: MINUTE 30, SECOND 45</t>
   </si>
 </sst>
 </file>
@@ -305,7 +326,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1"/>
@@ -320,6 +341,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
@@ -660,7 +682,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="525" row="3">
+  <wetp:taskpane dockstate="right" visibility="0" width="631" row="3">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -682,19 +704,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4323771-C859-F046-B681-A08AFC84A35B}">
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12.25" style="1" customWidth="1"/>
     <col min="2" max="3" width="11" style="1"/>
     <col min="4" max="4" width="11" style="8"/>
-    <col min="5" max="5" width="14.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5625" style="1" customWidth="1"/>
     <col min="6" max="8" width="11" style="1"/>
     <col min="9" max="9" width="37" style="1" customWidth="1"/>
     <col min="10" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -719,8 +741,9 @@
       <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="K1"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A2" s="1">
         <v>3</v>
       </c>
@@ -750,8 +773,9 @@
         <f>SECOND(D2)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="K2"/>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A3" s="1">
         <v>24</v>
       </c>
@@ -784,8 +808,9 @@
       <c r="I3" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="K3"/>
+    </row>
+    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A4" s="1">
         <v>16</v>
       </c>
@@ -818,8 +843,9 @@
       <c r="I4" s="5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="K4"/>
+    </row>
+    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A5" s="1">
         <v>3.1</v>
       </c>
@@ -852,8 +878,9 @@
       <c r="I5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="K5"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A6" s="1">
         <v>23</v>
       </c>
@@ -886,8 +913,9 @@
       <c r="I6" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="K6"/>
+    </row>
+    <row r="7" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="D7" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -912,7 +940,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>23</v>
       </c>
@@ -940,7 +968,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="B9" s="1">
         <v>23</v>
       </c>
@@ -968,7 +996,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="C10" s="1">
         <v>23</v>
       </c>
@@ -996,7 +1024,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>-1</v>
       </c>
@@ -1030,7 +1058,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <v>12</v>
       </c>
@@ -1064,7 +1092,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <v>13</v>
       </c>
@@ -1098,7 +1126,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <v>34</v>
       </c>
@@ -1132,7 +1160,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
         <v>10</v>
       </c>
@@ -1166,7 +1194,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
         <v>10</v>
       </c>
@@ -1490,23 +1518,23 @@
         <v>0</v>
       </c>
       <c r="D26" s="7">
-        <f>TIME(A26,B26,C26)</f>
+        <f t="shared" ref="D26:D38" si="42">TIME(A26,B26,C26)</f>
         <v>0</v>
       </c>
       <c r="E26" s="9">
-        <f>D26</f>
+        <f t="shared" ref="E26:E38" si="43">D26</f>
         <v>0</v>
       </c>
       <c r="F26" s="2">
-        <f>HOUR(D26)</f>
+        <f t="shared" ref="F26:F38" si="44">HOUR(D26)</f>
         <v>0</v>
       </c>
       <c r="G26" s="2">
-        <f>MINUTE(D26)</f>
+        <f t="shared" ref="G26:G38" si="45">MINUTE(D26)</f>
         <v>0</v>
       </c>
       <c r="H26" s="2">
-        <f>SECOND(D26)</f>
+        <f t="shared" ref="H26:H38" si="46">SECOND(D26)</f>
         <v>0</v>
       </c>
       <c r="I26" s="1" t="s">
@@ -1524,23 +1552,23 @@
         <v>1</v>
       </c>
       <c r="D27" s="7">
-        <f>TIME(A27,B27,C27)</f>
+        <f t="shared" si="42"/>
         <v>1.1574074074074073E-5</v>
       </c>
       <c r="E27" s="9">
-        <f>D27</f>
+        <f t="shared" si="43"/>
         <v>1.1574074074074073E-5</v>
       </c>
       <c r="F27" s="2">
-        <f>HOUR(D27)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="G27" s="2">
-        <f>MINUTE(D27)</f>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="H27" s="2">
-        <f>SECOND(D27)</f>
+        <f t="shared" si="46"/>
         <v>1</v>
       </c>
       <c r="I27" s="1" t="s">
@@ -1558,23 +1586,23 @@
         <v>59</v>
       </c>
       <c r="D28" s="7">
-        <f>TIME(A28,B28,C28)</f>
+        <f t="shared" si="42"/>
         <v>0.99998842592592596</v>
       </c>
       <c r="E28" s="9">
-        <f>D28</f>
+        <f t="shared" si="43"/>
         <v>0.99998842592592596</v>
       </c>
       <c r="F28" s="2">
-        <f>HOUR(D28)</f>
+        <f t="shared" si="44"/>
         <v>23</v>
       </c>
       <c r="G28" s="2">
-        <f>MINUTE(D28)</f>
+        <f t="shared" si="45"/>
         <v>59</v>
       </c>
       <c r="H28" s="2">
-        <f>SECOND(D28)</f>
+        <f t="shared" si="46"/>
         <v>59</v>
       </c>
       <c r="I28" s="1" t="s">
@@ -1592,23 +1620,23 @@
         <v>60</v>
       </c>
       <c r="D29" s="7">
-        <f>TIME(A29,B29,C29)</f>
+        <f t="shared" si="42"/>
         <v>0</v>
       </c>
       <c r="E29" s="9">
-        <f>D29</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="F29" s="2">
-        <f>HOUR(D29)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="G29" s="2">
-        <f>MINUTE(D29)</f>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="H29" s="2">
-        <f>SECOND(D29)</f>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="I29" s="1" t="s">
@@ -1626,23 +1654,23 @@
         <v>0</v>
       </c>
       <c r="D30" s="7">
-        <f>TIME(A30,B30,C30)</f>
+        <f t="shared" si="42"/>
         <v>0</v>
       </c>
       <c r="E30" s="9">
-        <f>D30</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="F30" s="2">
-        <f>HOUR(D30)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="G30" s="2">
-        <f>MINUTE(D30)</f>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="H30" s="2">
-        <f>SECOND(D30)</f>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="I30" s="1" t="s">
@@ -1660,23 +1688,23 @@
         <v>0</v>
       </c>
       <c r="D31" s="7">
-        <f>TIME(A31,B31,C31)</f>
+        <f t="shared" si="42"/>
         <v>0</v>
       </c>
       <c r="E31" s="9">
-        <f>D31</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="F31" s="2">
-        <f>HOUR(D31)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="G31" s="2">
-        <f>MINUTE(D31)</f>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="H31" s="2">
-        <f>SECOND(D31)</f>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="I31" s="1" t="s">
@@ -1694,23 +1722,23 @@
         <v>0</v>
       </c>
       <c r="D32" s="7">
-        <f>TIME(A32,B32,C32)</f>
+        <f t="shared" si="42"/>
         <v>0</v>
       </c>
       <c r="E32" s="9">
-        <f>D32</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="F32" s="2">
-        <f>HOUR(D32)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="G32" s="2">
-        <f>MINUTE(D32)</f>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="H32" s="2">
-        <f>SECOND(D32)</f>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="I32" s="1" t="s">
@@ -1728,23 +1756,23 @@
         <v>-1</v>
       </c>
       <c r="D33" s="7" t="e">
-        <f>TIME(A33,B33,C33)</f>
+        <f t="shared" si="42"/>
         <v>#NUM!</v>
       </c>
       <c r="E33" s="9" t="e">
-        <f>D33</f>
+        <f t="shared" si="43"/>
         <v>#NUM!</v>
       </c>
       <c r="F33" s="2" t="e">
-        <f>HOUR(D33)</f>
+        <f t="shared" si="44"/>
         <v>#NUM!</v>
       </c>
       <c r="G33" s="2" t="e">
-        <f>MINUTE(D33)</f>
+        <f t="shared" si="45"/>
         <v>#NUM!</v>
       </c>
       <c r="H33" s="2" t="e">
-        <f>SECOND(D33)</f>
+        <f t="shared" si="46"/>
         <v>#NUM!</v>
       </c>
       <c r="I33" s="1" t="s">
@@ -1762,23 +1790,23 @@
         <v>-1</v>
       </c>
       <c r="D34" s="7" t="e">
-        <f>TIME(A34,B34,C34)</f>
+        <f t="shared" si="42"/>
         <v>#NUM!</v>
       </c>
       <c r="E34" s="9" t="e">
-        <f>D34</f>
+        <f t="shared" si="43"/>
         <v>#NUM!</v>
       </c>
       <c r="F34" s="2" t="e">
-        <f>HOUR(D34)</f>
+        <f t="shared" si="44"/>
         <v>#NUM!</v>
       </c>
       <c r="G34" s="2" t="e">
-        <f>MINUTE(D34)</f>
+        <f t="shared" si="45"/>
         <v>#NUM!</v>
       </c>
       <c r="H34" s="2" t="e">
-        <f>SECOND(D34)</f>
+        <f t="shared" si="46"/>
         <v>#NUM!</v>
       </c>
       <c r="I34" s="1" t="s">
@@ -1796,23 +1824,23 @@
         <v>0</v>
       </c>
       <c r="D35" s="7" t="e">
-        <f>TIME(A35,B35,C35)</f>
+        <f t="shared" si="42"/>
         <v>#NUM!</v>
       </c>
       <c r="E35" s="9" t="e">
-        <f>D35</f>
+        <f t="shared" si="43"/>
         <v>#NUM!</v>
       </c>
       <c r="F35" s="2" t="e">
-        <f>HOUR(D35)</f>
+        <f t="shared" si="44"/>
         <v>#NUM!</v>
       </c>
       <c r="G35" s="2" t="e">
-        <f>MINUTE(D35)</f>
+        <f t="shared" si="45"/>
         <v>#NUM!</v>
       </c>
       <c r="H35" s="2" t="e">
-        <f>SECOND(D35)</f>
+        <f t="shared" si="46"/>
         <v>#NUM!</v>
       </c>
       <c r="I35" s="1" t="s">
@@ -1830,23 +1858,23 @@
         <v>0.49990000000000001</v>
       </c>
       <c r="D36" s="7">
-        <f>TIME(A36,B36,C36)</f>
+        <f t="shared" si="42"/>
         <v>4.2361111111111113E-2</v>
       </c>
       <c r="E36" s="9">
-        <f>D36</f>
+        <f t="shared" si="43"/>
         <v>4.2361111111111113E-2</v>
       </c>
       <c r="F36" s="2">
-        <f>HOUR(D36)</f>
+        <f t="shared" si="44"/>
         <v>1</v>
       </c>
       <c r="G36" s="2">
-        <f>MINUTE(D36)</f>
+        <f t="shared" si="45"/>
         <v>1</v>
       </c>
       <c r="H36" s="2">
-        <f>SECOND(D36)</f>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="I36" s="1" t="s">
@@ -1864,23 +1892,23 @@
         <v>0.5</v>
       </c>
       <c r="D37" s="7">
-        <f>TIME(A37,B37,C37)</f>
+        <f t="shared" si="42"/>
         <v>4.2361111111111113E-2</v>
       </c>
       <c r="E37" s="9">
-        <f>D37</f>
+        <f t="shared" si="43"/>
         <v>4.2361111111111113E-2</v>
       </c>
       <c r="F37" s="2">
-        <f>HOUR(D37)</f>
+        <f t="shared" si="44"/>
         <v>1</v>
       </c>
       <c r="G37" s="2">
-        <f>MINUTE(D37)</f>
+        <f t="shared" si="45"/>
         <v>1</v>
       </c>
       <c r="H37" s="2">
-        <f>SECOND(D37)</f>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="I37" s="1" t="s">
@@ -1898,23 +1926,23 @@
         <v>1.0000000000000001E-9</v>
       </c>
       <c r="D38" s="7">
-        <f>TIME(A38,B38,C38)</f>
+        <f t="shared" si="42"/>
         <v>0</v>
       </c>
       <c r="E38" s="9">
-        <f>D38</f>
+        <f t="shared" si="43"/>
         <v>0</v>
       </c>
       <c r="F38" s="2">
-        <f>HOUR(D38)</f>
+        <f t="shared" si="44"/>
         <v>0</v>
       </c>
       <c r="G38" s="2">
-        <f>MINUTE(D38)</f>
+        <f t="shared" si="45"/>
         <v>0</v>
       </c>
       <c r="H38" s="2">
-        <f>SECOND(D38)</f>
+        <f t="shared" si="46"/>
         <v>0</v>
       </c>
       <c r="I38" s="1" t="s">
@@ -1927,15 +1955,15 @@
         <v>45823.604687500003</v>
       </c>
       <c r="F40" s="2">
-        <f t="shared" ref="F40:F51" si="42">HOUR(E40)</f>
+        <f t="shared" ref="F40:F51" si="47">HOUR(E40)</f>
         <v>14</v>
       </c>
       <c r="G40" s="2">
-        <f t="shared" ref="G40:G51" si="43">MINUTE(E40)</f>
+        <f t="shared" ref="G40:G51" si="48">MINUTE(E40)</f>
         <v>30</v>
       </c>
       <c r="H40" s="2">
-        <f t="shared" ref="H40:H51" si="44">SECOND(E40)</f>
+        <f t="shared" ref="H40:H51" si="49">SECOND(E40)</f>
         <v>45</v>
       </c>
       <c r="I40" s="1" t="s">
@@ -1948,15 +1976,15 @@
         <v>45823</v>
       </c>
       <c r="F41" s="2">
-        <f t="shared" si="42"/>
+        <f t="shared" si="47"/>
         <v>0</v>
       </c>
       <c r="G41" s="2">
-        <f t="shared" si="43"/>
+        <f t="shared" si="48"/>
         <v>0</v>
       </c>
       <c r="H41" s="2">
-        <f t="shared" si="44"/>
+        <f t="shared" si="49"/>
         <v>0</v>
       </c>
       <c r="I41" s="1" t="s">
@@ -1968,15 +1996,15 @@
         <v>0</v>
       </c>
       <c r="F42" s="2">
-        <f t="shared" si="42"/>
+        <f t="shared" si="47"/>
         <v>0</v>
       </c>
       <c r="G42" s="2">
-        <f t="shared" si="43"/>
+        <f t="shared" si="48"/>
         <v>0</v>
       </c>
       <c r="H42" s="2">
-        <f t="shared" si="44"/>
+        <f t="shared" si="49"/>
         <v>0</v>
       </c>
       <c r="I42" s="1" t="s">
@@ -1988,15 +2016,15 @@
         <v>0.5</v>
       </c>
       <c r="F43" s="2">
-        <f t="shared" si="42"/>
+        <f t="shared" si="47"/>
         <v>12</v>
       </c>
       <c r="G43" s="2">
-        <f t="shared" si="43"/>
+        <f t="shared" si="48"/>
         <v>0</v>
       </c>
       <c r="H43" s="2">
-        <f t="shared" si="44"/>
+        <f t="shared" si="49"/>
         <v>0</v>
       </c>
       <c r="I43" s="1" t="s">
@@ -2008,15 +2036,15 @@
         <v>0.25</v>
       </c>
       <c r="F44" s="2">
-        <f t="shared" si="42"/>
+        <f t="shared" si="47"/>
         <v>6</v>
       </c>
       <c r="G44" s="2">
-        <f t="shared" si="43"/>
+        <f t="shared" si="48"/>
         <v>0</v>
       </c>
       <c r="H44" s="2">
-        <f t="shared" si="44"/>
+        <f t="shared" si="49"/>
         <v>0</v>
       </c>
       <c r="I44" s="1" t="s">
@@ -2028,15 +2056,15 @@
         <v>1.0000000010000001</v>
       </c>
       <c r="F45" s="2">
-        <f t="shared" si="42"/>
+        <f t="shared" si="47"/>
         <v>0</v>
       </c>
       <c r="G45" s="2">
-        <f t="shared" si="43"/>
+        <f t="shared" si="48"/>
         <v>0</v>
       </c>
       <c r="H45" s="2">
-        <f t="shared" si="44"/>
+        <f t="shared" si="49"/>
         <v>0</v>
       </c>
       <c r="I45" s="1" t="s">
@@ -2048,15 +2076,15 @@
         <v>1</v>
       </c>
       <c r="F46" s="2">
-        <f t="shared" si="42"/>
+        <f t="shared" si="47"/>
         <v>0</v>
       </c>
       <c r="G46" s="2">
-        <f t="shared" si="43"/>
+        <f t="shared" si="48"/>
         <v>0</v>
       </c>
       <c r="H46" s="2">
-        <f t="shared" si="44"/>
+        <f t="shared" si="49"/>
         <v>0</v>
       </c>
       <c r="I46" s="1" t="s">
@@ -2068,15 +2096,15 @@
         <v>-0.5</v>
       </c>
       <c r="F47" s="2" t="e">
-        <f t="shared" si="42"/>
+        <f t="shared" si="47"/>
         <v>#NUM!</v>
       </c>
       <c r="G47" s="2" t="e">
-        <f t="shared" si="43"/>
+        <f t="shared" si="48"/>
         <v>#NUM!</v>
       </c>
       <c r="H47" s="2" t="e">
-        <f t="shared" si="44"/>
+        <f t="shared" si="49"/>
         <v>#NUM!</v>
       </c>
       <c r="I47" s="1" t="s">
@@ -2088,15 +2116,15 @@
         <v>-1</v>
       </c>
       <c r="F48" s="2" t="e">
-        <f t="shared" si="42"/>
+        <f t="shared" si="47"/>
         <v>#NUM!</v>
       </c>
       <c r="G48" s="2" t="e">
-        <f t="shared" si="43"/>
+        <f t="shared" si="48"/>
         <v>#NUM!</v>
       </c>
       <c r="H48" s="2" t="e">
-        <f t="shared" si="44"/>
+        <f t="shared" si="49"/>
         <v>#NUM!</v>
       </c>
       <c r="I48" s="1" t="s">
@@ -2108,15 +2136,15 @@
         <v>-9.9999999999999995E-8</v>
       </c>
       <c r="F49" s="2" t="e">
-        <f t="shared" ref="F49" si="45">HOUR(E49)</f>
+        <f t="shared" ref="F49" si="50">HOUR(E49)</f>
         <v>#NUM!</v>
       </c>
       <c r="G49" s="2" t="e">
-        <f t="shared" ref="G49" si="46">MINUTE(E49)</f>
+        <f t="shared" ref="G49" si="51">MINUTE(E49)</f>
         <v>#NUM!</v>
       </c>
       <c r="H49" s="2" t="e">
-        <f t="shared" ref="H49" si="47">SECOND(E49)</f>
+        <f t="shared" ref="H49" si="52">SECOND(E49)</f>
         <v>#NUM!</v>
       </c>
       <c r="I49" s="10" t="s">
@@ -2128,15 +2156,15 @@
         <v>1</v>
       </c>
       <c r="F50" s="2">
-        <f t="shared" si="42"/>
+        <f t="shared" si="47"/>
         <v>0</v>
       </c>
       <c r="G50" s="2">
-        <f t="shared" si="43"/>
+        <f t="shared" si="48"/>
         <v>0</v>
       </c>
       <c r="H50" s="2">
-        <f t="shared" si="44"/>
+        <f t="shared" si="49"/>
         <v>0</v>
       </c>
       <c r="I50" s="1" t="s">
@@ -2149,23 +2177,170 @@
         <v>#N/A</v>
       </c>
       <c r="F51" s="2" t="e">
-        <f t="shared" si="42"/>
+        <f t="shared" si="47"/>
         <v>#N/A</v>
       </c>
       <c r="G51" s="2" t="e">
-        <f t="shared" si="43"/>
+        <f t="shared" si="48"/>
         <v>#N/A</v>
       </c>
       <c r="H51" s="2" t="e">
-        <f t="shared" si="44"/>
+        <f t="shared" si="49"/>
         <v>#N/A</v>
       </c>
       <c r="I51" s="1" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="52" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E52" s="1">
+        <v>0.52083333300000001</v>
+      </c>
+      <c r="F52" s="2">
+        <f t="shared" ref="F52:F53" si="53">HOUR(E52)</f>
+        <v>12</v>
+      </c>
+      <c r="G52" s="2">
+        <f t="shared" ref="G52:G53" si="54">MINUTE(E52)</f>
+        <v>30</v>
+      </c>
+      <c r="H52" s="2">
+        <f t="shared" ref="H52:H53" si="55">SECOND(E52)</f>
+        <v>0</v>
+      </c>
+      <c r="I52" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E53" s="12">
+        <f>12.5/24-0.0004/86400</f>
+        <v>0.52083332870370369</v>
+      </c>
+      <c r="F53" s="2">
+        <f>HOUR(E53)</f>
+        <v>12</v>
+      </c>
+      <c r="G53" s="2">
+        <f>MINUTE(E53)</f>
+        <v>30</v>
+      </c>
+      <c r="H53" s="2">
+        <f>SECOND(E53)</f>
+        <v>0</v>
+      </c>
+      <c r="I53" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="54" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E54" s="12">
+        <f>DATE(2025,6,15)+12.5/24-0.0004/86400</f>
+        <v>45823.520833328708</v>
+      </c>
+      <c r="F54" s="2">
+        <f>HOUR(E54)</f>
+        <v>12</v>
+      </c>
+      <c r="G54" s="2">
+        <f>MINUTE(E54)</f>
+        <v>30</v>
+      </c>
+      <c r="H54" s="2">
+        <f>SECOND(E54)</f>
+        <v>0</v>
+      </c>
+      <c r="I54" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E55" s="12">
+        <f>1/1440-0.0000000001</f>
+        <v>6.9444434444444444E-4</v>
+      </c>
+      <c r="F55" s="2">
+        <f>HOUR(E55)</f>
+        <v>0</v>
+      </c>
+      <c r="G55" s="2">
+        <f>MINUTE(E55)</f>
+        <v>1</v>
+      </c>
+      <c r="H55" s="2">
+        <f>SECOND(E55)</f>
+        <v>0</v>
+      </c>
+      <c r="I55" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="56" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E56" s="12">
+        <f>3/86400-0.000000001</f>
+        <v>3.472122222222222E-5</v>
+      </c>
+      <c r="F56" s="2">
+        <f>HOUR(E56)</f>
+        <v>0</v>
+      </c>
+      <c r="G56" s="2">
+        <f>MINUTE(E56)</f>
+        <v>0</v>
+      </c>
+      <c r="H56" s="2">
+        <f>SECOND(E56)</f>
+        <v>3</v>
+      </c>
+      <c r="I56" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="57" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E57" s="12">
+        <f>0.5+29.9996/86400</f>
+        <v>0.5003472175925926</v>
+      </c>
+      <c r="F57" s="2">
+        <f>HOUR(E57)</f>
+        <v>12</v>
+      </c>
+      <c r="G57" s="2">
+        <f>MINUTE(E57)</f>
+        <v>0</v>
+      </c>
+      <c r="H57" s="2">
+        <f>SECOND(E57)</f>
+        <v>30</v>
+      </c>
+      <c r="I57" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="58" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E58" s="12">
+        <f>TIME(14,30,45.999)</f>
+        <v>0.60468750000000004</v>
+      </c>
+      <c r="F58" s="2">
+        <f>HOUR(E58)</f>
+        <v>14</v>
+      </c>
+      <c r="G58" s="2">
+        <f>MINUTE(E58)</f>
+        <v>30</v>
+      </c>
+      <c r="H58" s="2">
+        <f>SECOND(E58)</f>
+        <v>45</v>
+      </c>
+      <c r="I58" s="10" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update: improve testing for TIME, HOUR, MINUTE, SECOND (#1456)
* update: extend xlsx tests and argument unit tests for TIME, HOUR, MINUTE, SECOND

* update: add xlsx tests for TIME, HOUR, MINUTE, SECOND

* update: add unit tests for TIME, HOUR, MINUTE, SECOND

* update: add more test cases that cover #1432
</commit_message>
<xml_diff>
--- a/xlsx/tests/calc_tests/DATE_AND_TIME/TIME_HOUR_MINUTE_SECOND.xlsx
+++ b/xlsx/tests/calc_tests/DATE_AND_TIME/TIME_HOUR_MINUTE_SECOND.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29429"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nhatcher/Documents/Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elsam\Documents\IronCalc stuff\my_calc_tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBC0634F-134E-41A2-B667-6435048C259E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC112A6F-ADF2-48B2-AF26-281DCF89B185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33600" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{F5EF1803-C89D-8542-8C3F-E05EFF447D52}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{F5EF1803-C89D-8542-8C3F-E05EFF447D52}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,8 +35,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="57">
   <si>
     <t>HOUR</t>
   </si>
@@ -111,6 +133,102 @@
   </si>
   <si>
     <t>Boolean as input</t>
+  </si>
+  <si>
+    <t>All arguments zero</t>
+  </si>
+  <si>
+    <t>Smallest non-zero time</t>
+  </si>
+  <si>
+    <t>Largest time within one day</t>
+  </si>
+  <si>
+    <t>Seconds roll over into the next day</t>
+  </si>
+  <si>
+    <t>Minutes equal to exactly one day</t>
+  </si>
+  <si>
+    <t>Hours equal to exactly one day</t>
+  </si>
+  <si>
+    <t>Hours equal to exactly two days</t>
+  </si>
+  <si>
+    <t>All arguments negative</t>
+  </si>
+  <si>
+    <t>Negative seconds from midnight</t>
+  </si>
+  <si>
+    <t>Negative minutes from midnight</t>
+  </si>
+  <si>
+    <t>Seconds fraction rounds down</t>
+  </si>
+  <si>
+    <t>Seconds fraction at the rounding midpoint</t>
+  </si>
+  <si>
+    <t>All arguments just above zero</t>
+  </si>
+  <si>
+    <t>Date with a time portion</t>
+  </si>
+  <si>
+    <t>Whole date, no time portion</t>
+  </si>
+  <si>
+    <t>Serial 0</t>
+  </si>
+  <si>
+    <t>Serial 0.5, exactly midday</t>
+  </si>
+  <si>
+    <t>Serial 0.25, 6am</t>
+  </si>
+  <si>
+    <t>Serial 1, exactly one day</t>
+  </si>
+  <si>
+    <t>Negative serial</t>
+  </si>
+  <si>
+    <t>Negative whole serial</t>
+  </si>
+  <si>
+    <t>Serial just above one whole day</t>
+  </si>
+  <si>
+    <t>Boolean TRUE</t>
+  </si>
+  <si>
+    <t>Error propagation mixed</t>
+  </si>
+  <si>
+    <t>Negative near zero</t>
+  </si>
+  <si>
+    <t>Time 12:29:59.99997 as fractional</t>
+  </si>
+  <si>
+    <t>Time 0.4 ms under 12:30:00 rounds up: MINUTE 30, SECOND 0</t>
+  </si>
+  <si>
+    <t>Same as above with a date portion: MINUTE 30, SECOND 0</t>
+  </si>
+  <si>
+    <t>Arithmetic result just under 00:01:00: MINUTE 1, SECOND 0</t>
+  </si>
+  <si>
+    <t>Arithmetic result just under 3 s: MINUTE 0, SECOND 3</t>
+  </si>
+  <si>
+    <t>12:00:29.9996 rounds up to 30 s: MINUTE 0, SECOND 30</t>
+  </si>
+  <si>
+    <t>Existing behaviour kept: MINUTE 30, SECOND 45</t>
   </si>
 </sst>
 </file>
@@ -118,10 +236,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="165" formatCode="0.0000000000"/>
-    <numFmt numFmtId="166" formatCode="h:mm:ss;@"/>
+    <numFmt numFmtId="164" formatCode="0.0000000000"/>
+    <numFmt numFmtId="165" formatCode="h:mm:ss;@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -153,6 +271,18 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -196,18 +326,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Calculation" xfId="1" builtinId="22"/>
@@ -215,6 +349,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFEDDAB1"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -541,21 +680,43 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="631" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{86F010F7-E038-4299-9ABC-6B7FD165E119}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;759a215b-68d0-4a32-b792-08a4fe5196a6&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4323771-C859-F046-B681-A08AFC84A35B}">
-  <dimension ref="A1:I36"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="A1:K58"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12.25" style="1" customWidth="1"/>
     <col min="2" max="3" width="11" style="1"/>
     <col min="4" max="4" width="11" style="8"/>
-    <col min="5" max="5" width="14.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5625" style="1" customWidth="1"/>
     <col min="6" max="8" width="11" style="1"/>
     <col min="9" max="9" width="37" style="1" customWidth="1"/>
     <col min="10" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.75">
+    <row r="1" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -580,8 +741,9 @@
       <c r="H1" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="K1"/>
+    </row>
+    <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A2" s="1">
         <v>3</v>
       </c>
@@ -611,8 +773,9 @@
         <f>SECOND(D2)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:9">
+      <c r="K2"/>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A3" s="1">
         <v>24</v>
       </c>
@@ -645,8 +808,9 @@
       <c r="I3" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:9">
+      <c r="K3"/>
+    </row>
+    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A4" s="1">
         <v>16</v>
       </c>
@@ -661,7 +825,7 @@
         <v>0.70861111111111108</v>
       </c>
       <c r="E4" s="4">
-        <f t="shared" ref="E4:E26" si="1">D4</f>
+        <f t="shared" ref="E4:E24" si="1">D4</f>
         <v>0.70861111111111108</v>
       </c>
       <c r="F4" s="2">
@@ -679,8 +843,9 @@
       <c r="I4" s="5" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:9">
+      <c r="K4"/>
+    </row>
+    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A5" s="1">
         <v>3.1</v>
       </c>
@@ -713,8 +878,9 @@
       <c r="I5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:9">
+      <c r="K5"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.5">
       <c r="A6" s="1">
         <v>23</v>
       </c>
@@ -747,8 +913,9 @@
       <c r="I6" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:9">
+      <c r="K6"/>
+    </row>
+    <row r="7" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="D7" s="7">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -773,7 +940,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A8" s="1">
         <v>23</v>
       </c>
@@ -801,7 +968,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="B9" s="1">
         <v>23</v>
       </c>
@@ -829,7 +996,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="C10" s="1">
         <v>23</v>
       </c>
@@ -857,7 +1024,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A11" s="1">
         <v>-1</v>
       </c>
@@ -891,7 +1058,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A12" s="1">
         <v>12</v>
       </c>
@@ -925,7 +1092,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A13" s="1">
         <v>13</v>
       </c>
@@ -959,7 +1126,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A14" s="1">
         <v>34</v>
       </c>
@@ -993,7 +1160,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A15" s="1">
         <v>10</v>
       </c>
@@ -1027,7 +1194,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:11" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A16" s="1">
         <v>10</v>
       </c>
@@ -1061,7 +1228,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A17" s="1">
         <v>32767</v>
       </c>
@@ -1095,7 +1262,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A18" s="1" t="e">
         <f>1/0</f>
         <v>#DIV/0!</v>
@@ -1130,19 +1297,19 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A19" s="1">
         <v>1</v>
       </c>
       <c r="B19" s="1" t="e">
-        <f t="shared" ref="B19:C20" si="28">1/0</f>
+        <f t="shared" ref="B19:C21" si="28">1/0</f>
         <v>#DIV/0!</v>
       </c>
       <c r="C19" s="1">
         <v>3</v>
       </c>
       <c r="D19" s="7" t="e">
-        <f t="shared" ref="D19:D26" si="29">TIME(A19,B19,C19)</f>
+        <f t="shared" ref="D19:D24" si="29">TIME(A19,B19,C19)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="E19" s="4" t="e">
@@ -1150,22 +1317,22 @@
         <v>#DIV/0!</v>
       </c>
       <c r="F19" s="2" t="e">
-        <f t="shared" ref="F19:F23" si="30">HOUR(D19)</f>
+        <f t="shared" ref="F19:F20" si="30">HOUR(D19)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="G19" s="2" t="e">
-        <f t="shared" ref="G19:G23" si="31">MINUTE(D19)</f>
+        <f t="shared" ref="G19:G20" si="31">MINUTE(D19)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="H19" s="2" t="e">
-        <f t="shared" ref="H19:H23" si="32">SECOND(D19)</f>
+        <f t="shared" ref="H19:H20" si="32">SECOND(D19)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A20" s="1">
         <v>1</v>
       </c>
@@ -1200,224 +1367,980 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A21" s="1" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="B21" s="1">
-        <v>2</v>
-      </c>
-      <c r="C21" s="1">
-        <v>3</v>
+      <c r="B21" s="1" t="e">
+        <f t="shared" si="28"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="C21" s="1" t="e" cm="1">
+        <f t="array" aca="1" ref="C21" ca="1">hello()</f>
+        <v>#NAME?</v>
       </c>
       <c r="D21" s="7" t="e">
+        <f ca="1">TIME(A21,B21,C21)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E21" s="4" t="e">
+        <f ca="1">D21</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F21" s="2" t="e">
+        <f ca="1">HOUR(D21)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G21" s="2" t="e">
+        <f ca="1">MINUTE(D21)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H21" s="2" t="e">
+        <f ca="1">SECOND(D21)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D22" s="7" t="e">
         <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="E21" s="4" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E22" s="4" t="e">
         <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="F21" s="2" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="G21" s="2" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H21" s="2" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" s="1">
-        <v>1</v>
-      </c>
-      <c r="B22" s="1" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F22" s="2" t="e">
+        <f t="shared" ref="F22" si="33">HOUR(D22)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G22" s="2" t="e">
+        <f t="shared" ref="G22" si="34">MINUTE(D22)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H22" s="2" t="e">
+        <f t="shared" ref="H22" si="35">SECOND(D22)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A23" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D23" s="7" t="e">
+        <f t="shared" si="29"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="E23" s="4" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
+      <c r="F23" s="2" t="e">
+        <f t="shared" ref="F23" si="36">HOUR(D23)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="G23" s="2" t="e">
+        <f t="shared" ref="G23" si="37">MINUTE(D23)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="H23" s="2" t="e">
+        <f t="shared" ref="H23" si="38">SECOND(D23)</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A24" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="B24" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="C24" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="D24" s="7">
+        <f t="shared" si="29"/>
+        <v>4.1678240740740738E-2</v>
+      </c>
+      <c r="E24" s="4">
+        <f t="shared" si="1"/>
+        <v>4.1678240740740738E-2</v>
+      </c>
+      <c r="F24" s="2">
+        <f t="shared" ref="F24" si="39">HOUR(D24)</f>
+        <v>1</v>
+      </c>
+      <c r="G24" s="2">
+        <f t="shared" ref="G24" si="40">MINUTE(D24)</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="2">
+        <f t="shared" ref="H24" si="41">SECOND(D24)</f>
+        <v>1</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="14.25" x14ac:dyDescent="0.45"/>
+    <row r="26" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A26" s="1">
+        <v>0</v>
+      </c>
+      <c r="B26" s="1">
+        <v>0</v>
+      </c>
+      <c r="C26" s="1">
+        <v>0</v>
+      </c>
+      <c r="D26" s="7">
+        <f t="shared" ref="D26:D38" si="42">TIME(A26,B26,C26)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="9">
+        <f t="shared" ref="E26:E38" si="43">D26</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="2">
+        <f t="shared" ref="F26:F38" si="44">HOUR(D26)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="2">
+        <f t="shared" ref="G26:G38" si="45">MINUTE(D26)</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="2">
+        <f t="shared" ref="H26:H38" si="46">SECOND(D26)</f>
+        <v>0</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A27" s="1">
+        <v>0</v>
+      </c>
+      <c r="B27" s="1">
+        <v>0</v>
+      </c>
+      <c r="C27" s="1">
+        <v>1</v>
+      </c>
+      <c r="D27" s="7">
+        <f t="shared" si="42"/>
+        <v>1.1574074074074073E-5</v>
+      </c>
+      <c r="E27" s="9">
+        <f t="shared" si="43"/>
+        <v>1.1574074074074073E-5</v>
+      </c>
+      <c r="F27" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G27" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H27" s="2">
+        <f t="shared" si="46"/>
+        <v>1</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A28" s="1">
+        <v>23</v>
+      </c>
+      <c r="B28" s="1">
+        <v>59</v>
+      </c>
+      <c r="C28" s="1">
+        <v>59</v>
+      </c>
+      <c r="D28" s="7">
+        <f t="shared" si="42"/>
+        <v>0.99998842592592596</v>
+      </c>
+      <c r="E28" s="9">
+        <f t="shared" si="43"/>
+        <v>0.99998842592592596</v>
+      </c>
+      <c r="F28" s="2">
+        <f t="shared" si="44"/>
+        <v>23</v>
+      </c>
+      <c r="G28" s="2">
+        <f t="shared" si="45"/>
+        <v>59</v>
+      </c>
+      <c r="H28" s="2">
+        <f t="shared" si="46"/>
+        <v>59</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="14.25" x14ac:dyDescent="0.45">
+      <c r="A29" s="1">
+        <v>23</v>
+      </c>
+      <c r="B29" s="1">
+        <v>59</v>
+      </c>
+      <c r="C29" s="1">
+        <v>60</v>
+      </c>
+      <c r="D29" s="7">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="E29" s="9">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="F29" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G29" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H29" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A30" s="1">
+        <v>0</v>
+      </c>
+      <c r="B30" s="1">
+        <v>1440</v>
+      </c>
+      <c r="C30" s="1">
+        <v>0</v>
+      </c>
+      <c r="D30" s="7">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="E30" s="9">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="F30" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G30" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H30" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I30" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A31" s="1">
+        <v>24</v>
+      </c>
+      <c r="B31" s="1">
+        <v>0</v>
+      </c>
+      <c r="C31" s="1">
+        <v>0</v>
+      </c>
+      <c r="D31" s="7">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="E31" s="9">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="F31" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G31" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H31" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A32" s="1">
+        <v>48</v>
+      </c>
+      <c r="B32" s="1">
+        <v>0</v>
+      </c>
+      <c r="C32" s="1">
+        <v>0</v>
+      </c>
+      <c r="D32" s="7">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="E32" s="9">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="F32" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G32" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H32" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="1">
+        <v>-1</v>
+      </c>
+      <c r="B33" s="1">
+        <v>-1</v>
+      </c>
+      <c r="C33" s="1">
+        <v>-1</v>
+      </c>
+      <c r="D33" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E33" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F33" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G33" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H33" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A34" s="1">
+        <v>0</v>
+      </c>
+      <c r="B34" s="1">
+        <v>0</v>
+      </c>
+      <c r="C34" s="1">
+        <v>-1</v>
+      </c>
+      <c r="D34" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E34" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F34" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G34" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H34" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A35" s="1">
+        <v>0</v>
+      </c>
+      <c r="B35" s="1">
+        <v>-1</v>
+      </c>
+      <c r="C35" s="1">
+        <v>0</v>
+      </c>
+      <c r="D35" s="7" t="e">
+        <f t="shared" si="42"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="E35" s="9" t="e">
+        <f t="shared" si="43"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="F35" s="2" t="e">
+        <f t="shared" si="44"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G35" s="2" t="e">
+        <f t="shared" si="45"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H35" s="2" t="e">
+        <f t="shared" si="46"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A36" s="1">
+        <v>1</v>
+      </c>
+      <c r="B36" s="1">
+        <v>1</v>
+      </c>
+      <c r="C36" s="1">
+        <v>0.49990000000000001</v>
+      </c>
+      <c r="D36" s="7">
+        <f t="shared" si="42"/>
+        <v>4.2361111111111113E-2</v>
+      </c>
+      <c r="E36" s="9">
+        <f t="shared" si="43"/>
+        <v>4.2361111111111113E-2</v>
+      </c>
+      <c r="F36" s="2">
+        <f t="shared" si="44"/>
+        <v>1</v>
+      </c>
+      <c r="G36" s="2">
+        <f t="shared" si="45"/>
+        <v>1</v>
+      </c>
+      <c r="H36" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A37" s="1">
+        <v>1</v>
+      </c>
+      <c r="B37" s="1">
+        <v>1</v>
+      </c>
+      <c r="C37" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="D37" s="7">
+        <f t="shared" si="42"/>
+        <v>4.2361111111111113E-2</v>
+      </c>
+      <c r="E37" s="9">
+        <f t="shared" si="43"/>
+        <v>4.2361111111111113E-2</v>
+      </c>
+      <c r="F37" s="2">
+        <f t="shared" si="44"/>
+        <v>1</v>
+      </c>
+      <c r="G37" s="2">
+        <f t="shared" si="45"/>
+        <v>1</v>
+      </c>
+      <c r="H37" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A38" s="1">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="B38" s="1">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="C38" s="1">
+        <v>1.0000000000000001E-9</v>
+      </c>
+      <c r="D38" s="7">
+        <f t="shared" si="42"/>
+        <v>0</v>
+      </c>
+      <c r="E38" s="9">
+        <f t="shared" si="43"/>
+        <v>0</v>
+      </c>
+      <c r="F38" s="2">
+        <f t="shared" si="44"/>
+        <v>0</v>
+      </c>
+      <c r="G38" s="2">
+        <f t="shared" si="45"/>
+        <v>0</v>
+      </c>
+      <c r="H38" s="2">
+        <f t="shared" si="46"/>
+        <v>0</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E40" s="1">
+        <f>DATE(2025,6,15)+TIME(14,30,45)</f>
+        <v>45823.604687500003</v>
+      </c>
+      <c r="F40" s="2">
+        <f t="shared" ref="F40:F51" si="47">HOUR(E40)</f>
+        <v>14</v>
+      </c>
+      <c r="G40" s="2">
+        <f t="shared" ref="G40:G51" si="48">MINUTE(E40)</f>
+        <v>30</v>
+      </c>
+      <c r="H40" s="2">
+        <f t="shared" ref="H40:H51" si="49">SECOND(E40)</f>
+        <v>45</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E41" s="1">
+        <f>DATE(2025,6,15)</f>
+        <v>45823</v>
+      </c>
+      <c r="F41" s="2">
+        <f t="shared" si="47"/>
+        <v>0</v>
+      </c>
+      <c r="G41" s="2">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="H41" s="2">
+        <f t="shared" si="49"/>
+        <v>0</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E42" s="1">
+        <v>0</v>
+      </c>
+      <c r="F42" s="2">
+        <f t="shared" si="47"/>
+        <v>0</v>
+      </c>
+      <c r="G42" s="2">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="H42" s="2">
+        <f t="shared" si="49"/>
+        <v>0</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E43" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="F43" s="2">
+        <f t="shared" si="47"/>
+        <v>12</v>
+      </c>
+      <c r="G43" s="2">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="H43" s="2">
+        <f t="shared" si="49"/>
+        <v>0</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E44" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="F44" s="2">
+        <f t="shared" si="47"/>
+        <v>6</v>
+      </c>
+      <c r="G44" s="2">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="H44" s="2">
+        <f t="shared" si="49"/>
+        <v>0</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E45" s="1">
+        <v>1.0000000010000001</v>
+      </c>
+      <c r="F45" s="2">
+        <f t="shared" si="47"/>
+        <v>0</v>
+      </c>
+      <c r="G45" s="2">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="H45" s="2">
+        <f t="shared" si="49"/>
+        <v>0</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E46" s="1">
+        <v>1</v>
+      </c>
+      <c r="F46" s="2">
+        <f t="shared" si="47"/>
+        <v>0</v>
+      </c>
+      <c r="G46" s="2">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="H46" s="2">
+        <f t="shared" si="49"/>
+        <v>0</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E47" s="1">
+        <v>-0.5</v>
+      </c>
+      <c r="F47" s="2" t="e">
+        <f t="shared" si="47"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G47" s="2" t="e">
+        <f t="shared" si="48"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H47" s="2" t="e">
+        <f t="shared" si="49"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E48" s="1">
+        <v>-1</v>
+      </c>
+      <c r="F48" s="2" t="e">
+        <f t="shared" si="47"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="G48" s="2" t="e">
+        <f t="shared" si="48"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="H48" s="2" t="e">
+        <f t="shared" si="49"/>
+        <v>#NUM!</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="49" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E49" s="11">
+        <v>-9.9999999999999995E-8</v>
+      </c>
+      <c r="F49" s="2" t="e">
+        <f t="shared" ref="F49" si="50">HOUR(E49)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="G49" s="2" t="e">
+        <f t="shared" ref="G49" si="51">MINUTE(E49)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="H49" s="2" t="e">
+        <f t="shared" ref="H49" si="52">SECOND(E49)</f>
+        <v>#NUM!</v>
+      </c>
+      <c r="I49" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E50" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="F50" s="2">
+        <f t="shared" si="47"/>
+        <v>0</v>
+      </c>
+      <c r="G50" s="2">
+        <f t="shared" si="48"/>
+        <v>0</v>
+      </c>
+      <c r="H50" s="2">
+        <f t="shared" si="49"/>
+        <v>0</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="51" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E51" s="1" t="e">
         <f>NA()</f>
         <v>#N/A</v>
       </c>
-      <c r="C22" s="1">
+      <c r="F51" s="2" t="e">
+        <f t="shared" si="47"/>
+        <v>#N/A</v>
+      </c>
+      <c r="G51" s="2" t="e">
+        <f t="shared" si="48"/>
+        <v>#N/A</v>
+      </c>
+      <c r="H51" s="2" t="e">
+        <f t="shared" si="49"/>
+        <v>#N/A</v>
+      </c>
+      <c r="I51" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="52" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E52" s="1">
+        <v>0.52083333300000001</v>
+      </c>
+      <c r="F52" s="2">
+        <f t="shared" ref="F52:F53" si="53">HOUR(E52)</f>
+        <v>12</v>
+      </c>
+      <c r="G52" s="2">
+        <f t="shared" ref="G52:G53" si="54">MINUTE(E52)</f>
+        <v>30</v>
+      </c>
+      <c r="H52" s="2">
+        <f t="shared" ref="H52:H53" si="55">SECOND(E52)</f>
+        <v>0</v>
+      </c>
+      <c r="I52" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="53" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E53" s="12">
+        <f>12.5/24-0.0004/86400</f>
+        <v>0.52083332870370369</v>
+      </c>
+      <c r="F53" s="2">
+        <f>HOUR(E53)</f>
+        <v>12</v>
+      </c>
+      <c r="G53" s="2">
+        <f>MINUTE(E53)</f>
+        <v>30</v>
+      </c>
+      <c r="H53" s="2">
+        <f>SECOND(E53)</f>
+        <v>0</v>
+      </c>
+      <c r="I53" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="54" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E54" s="12">
+        <f>DATE(2025,6,15)+12.5/24-0.0004/86400</f>
+        <v>45823.520833328708</v>
+      </c>
+      <c r="F54" s="2">
+        <f>HOUR(E54)</f>
+        <v>12</v>
+      </c>
+      <c r="G54" s="2">
+        <f>MINUTE(E54)</f>
+        <v>30</v>
+      </c>
+      <c r="H54" s="2">
+        <f>SECOND(E54)</f>
+        <v>0</v>
+      </c>
+      <c r="I54" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E55" s="12">
+        <f>1/1440-0.0000000001</f>
+        <v>6.9444434444444444E-4</v>
+      </c>
+      <c r="F55" s="2">
+        <f>HOUR(E55)</f>
+        <v>0</v>
+      </c>
+      <c r="G55" s="2">
+        <f>MINUTE(E55)</f>
+        <v>1</v>
+      </c>
+      <c r="H55" s="2">
+        <f>SECOND(E55)</f>
+        <v>0</v>
+      </c>
+      <c r="I55" s="10" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="56" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E56" s="12">
+        <f>3/86400-0.000000001</f>
+        <v>3.472122222222222E-5</v>
+      </c>
+      <c r="F56" s="2">
+        <f>HOUR(E56)</f>
+        <v>0</v>
+      </c>
+      <c r="G56" s="2">
+        <f>MINUTE(E56)</f>
+        <v>0</v>
+      </c>
+      <c r="H56" s="2">
+        <f>SECOND(E56)</f>
         <v>3</v>
       </c>
-      <c r="D22" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="E22" s="4" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="F22" s="2" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="G22" s="2" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H22" s="2" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I22" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" s="1">
-        <v>1</v>
-      </c>
-      <c r="B23" s="1">
-        <v>2</v>
-      </c>
-      <c r="C23" s="1" t="e">
-        <f>NA()</f>
-        <v>#N/A</v>
-      </c>
-      <c r="D23" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#N/A</v>
-      </c>
-      <c r="E23" s="4" t="e">
-        <f t="shared" si="1"/>
-        <v>#N/A</v>
-      </c>
-      <c r="F23" s="2" t="e">
-        <f t="shared" si="30"/>
-        <v>#N/A</v>
-      </c>
-      <c r="G23" s="2" t="e">
-        <f t="shared" si="31"/>
-        <v>#N/A</v>
-      </c>
-      <c r="H23" s="2" t="e">
-        <f t="shared" si="32"/>
-        <v>#N/A</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D24" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E24" s="4" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F24" s="2" t="e">
-        <f t="shared" ref="F24" si="33">HOUR(D24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G24" s="2" t="e">
-        <f t="shared" ref="G24" si="34">MINUTE(D24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H24" s="2" t="e">
-        <f t="shared" ref="H24" si="35">SECOND(D24)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D25" s="7" t="e">
-        <f t="shared" si="29"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E25" s="4" t="e">
-        <f t="shared" si="1"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F25" s="2" t="e">
-        <f t="shared" ref="F25" si="36">HOUR(D25)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G25" s="2" t="e">
-        <f t="shared" ref="G25" si="37">MINUTE(D25)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H25" s="2" t="e">
-        <f t="shared" ref="H25" si="38">SECOND(D25)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="A26" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="B26" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="C26" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="D26" s="7">
-        <f t="shared" si="29"/>
-        <v>4.1678240740740738E-2</v>
-      </c>
-      <c r="E26" s="4">
-        <f t="shared" si="1"/>
-        <v>4.1678240740740738E-2</v>
-      </c>
-      <c r="F26" s="2">
-        <f t="shared" ref="F26" si="39">HOUR(D26)</f>
-        <v>1</v>
-      </c>
-      <c r="G26" s="2">
-        <f t="shared" ref="G26" si="40">MINUTE(D26)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="2">
-        <f t="shared" ref="H26" si="41">SECOND(D26)</f>
-        <v>1</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9"/>
-    <row r="28" spans="1:9"/>
-    <row r="29" spans="1:9"/>
-    <row r="30" spans="1:9"/>
-    <row r="31" spans="1:9"/>
-    <row r="32" spans="1:9"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
+      <c r="I56" s="10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="57" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E57" s="12">
+        <f>0.5+29.9996/86400</f>
+        <v>0.5003472175925926</v>
+      </c>
+      <c r="F57" s="2">
+        <f>HOUR(E57)</f>
+        <v>12</v>
+      </c>
+      <c r="G57" s="2">
+        <f>MINUTE(E57)</f>
+        <v>0</v>
+      </c>
+      <c r="H57" s="2">
+        <f>SECOND(E57)</f>
+        <v>30</v>
+      </c>
+      <c r="I57" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="58" spans="5:9" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="E58" s="12">
+        <f>TIME(14,30,45.999)</f>
+        <v>0.60468750000000004</v>
+      </c>
+      <c r="F58" s="2">
+        <f>HOUR(E58)</f>
+        <v>14</v>
+      </c>
+      <c r="G58" s="2">
+        <f>MINUTE(E58)</f>
+        <v>30</v>
+      </c>
+      <c r="H58" s="2">
+        <f>SECOND(E58)</f>
+        <v>45</v>
+      </c>
+      <c r="I58" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>